<commit_message>
Regenerate all outputs from the current pipeline
Full re-run of Run_All.R. Picks up Tables 2 & 3 (the HT4/HT6 multivariable
regressions for NRS and SOWS, in both .xlsx and publication .docx/.html),
the config-caching fix -- which is what lets the figure styling below
actually take effect without an R restart -- and the enlarged figure text,
thicker points/lines, and per-panel facet axis rules, which is why every
.png/.tiff/.docx composite is touched.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/New_Outputs/Figure_StatsBox_Placement_Audit.xlsx
+++ b/New_Outputs/Figure_StatsBox_Placement_Audit.xlsx
@@ -142,25 +142,25 @@
     <t>Fig1_PC3_HT1A_Only</t>
   </si>
   <si>
+    <t>Fig1_PC3_HT1A_Only_overlay</t>
+  </si>
+  <si>
+    <t>Fig1_SOWS_HT1A_Only</t>
+  </si>
+  <si>
+    <t>Fig1_SOWS_HT1A_Only_overlay</t>
+  </si>
+  <si>
+    <t>Fig1_NRS_HT2A_Only</t>
+  </si>
+  <si>
+    <t>Fig1_NRS_HT2A_Only_overlay</t>
+  </si>
+  <si>
+    <t>Fig1_PC1_HT2A_Only</t>
+  </si>
+  <si>
     <t>bottomright</t>
-  </si>
-  <si>
-    <t>Fig1_PC3_HT1A_Only_overlay</t>
-  </si>
-  <si>
-    <t>Fig1_SOWS_HT1A_Only</t>
-  </si>
-  <si>
-    <t>Fig1_SOWS_HT1A_Only_overlay</t>
-  </si>
-  <si>
-    <t>Fig1_NRS_HT2A_Only</t>
-  </si>
-  <si>
-    <t>Fig1_NRS_HT2A_Only_overlay</t>
-  </si>
-  <si>
-    <t>Fig1_PC1_HT2A_Only</t>
   </si>
   <si>
     <t>Fig1_PC1_HT2A_Only_overlay</t>
@@ -891,16 +891,16 @@
         <v>0</v>
       </c>
       <c r="F2">
-        <v>1.62290249796904</v>
+        <v>1.549828320424181</v>
       </c>
       <c r="G2">
         <v>0</v>
       </c>
       <c r="H2">
-        <v>0.547988865787772</v>
+        <v>0.5391863577225988</v>
       </c>
       <c r="I2">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -920,16 +920,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>1.62290249796904</v>
+        <v>1.549828320424181</v>
       </c>
       <c r="G3">
         <v>0</v>
       </c>
       <c r="H3">
-        <v>0.547988865787772</v>
+        <v>0.5391863577225988</v>
       </c>
       <c r="I3">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -955,10 +955,10 @@
         <v>0</v>
       </c>
       <c r="H4">
-        <v>0.6377276726032395</v>
+        <v>0.6272881609575219</v>
       </c>
       <c r="I4">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -984,10 +984,10 @@
         <v>0</v>
       </c>
       <c r="H5">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I5">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -1013,10 +1013,10 @@
         <v>0</v>
       </c>
       <c r="H6">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I6">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -1042,10 +1042,10 @@
         <v>0</v>
       </c>
       <c r="H7">
-        <v>0.607661787116463</v>
+        <v>0.592782893328202</v>
       </c>
       <c r="I7">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -1065,16 +1065,16 @@
         <v>0</v>
       </c>
       <c r="F8">
-        <v>0.7266560749816646</v>
+        <v>0.6939370452779632</v>
       </c>
       <c r="G8">
         <v>0</v>
       </c>
       <c r="H8">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I8">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -1094,16 +1094,16 @@
         <v>0</v>
       </c>
       <c r="F9">
-        <v>0.7266560749816646</v>
+        <v>0.6939370452779632</v>
       </c>
       <c r="G9">
         <v>0</v>
       </c>
       <c r="H9">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I9">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -1123,16 +1123,16 @@
         <v>0</v>
       </c>
       <c r="F10">
-        <v>0.5589989523206498</v>
+        <v>0.530839023295139</v>
       </c>
       <c r="G10">
         <v>0</v>
       </c>
       <c r="H10">
-        <v>0.6038451386425255</v>
+        <v>0.5899789573712763</v>
       </c>
       <c r="I10">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -1158,10 +1158,10 @@
         <v>0</v>
       </c>
       <c r="H11">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I11">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -1172,7 +1172,7 @@
         <v>12</v>
       </c>
       <c r="C12" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="D12">
         <v>0</v>
@@ -1187,10 +1187,10 @@
         <v>0</v>
       </c>
       <c r="H12">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I12">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -1216,10 +1216,10 @@
         <v>0</v>
       </c>
       <c r="H13">
-        <v>0.6038451386425255</v>
+        <v>0.5899789573712763</v>
       </c>
       <c r="I13">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -1245,10 +1245,10 @@
         <v>0</v>
       </c>
       <c r="H14">
-        <v>0.5597192620311737</v>
+        <v>0.5512173913874463</v>
       </c>
       <c r="I14">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="15" spans="1:9">
@@ -1274,10 +1274,10 @@
         <v>0</v>
       </c>
       <c r="H15">
-        <v>0.5597192620311737</v>
+        <v>0.5512173913874463</v>
       </c>
       <c r="I15">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="16" spans="1:9">
@@ -1303,10 +1303,10 @@
         <v>0</v>
       </c>
       <c r="H16">
-        <v>0.6352144220446534</v>
+        <v>0.6251092030567968</v>
       </c>
       <c r="I16">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="17" spans="1:9">
@@ -1326,16 +1326,16 @@
         <v>0</v>
       </c>
       <c r="F17">
-        <v>1.62290249796904</v>
+        <v>1.549828320424181</v>
       </c>
       <c r="G17">
         <v>0</v>
       </c>
       <c r="H17">
-        <v>0.5236828282628889</v>
+        <v>0.5147706092489056</v>
       </c>
       <c r="I17">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="18" spans="1:9">
@@ -1355,16 +1355,16 @@
         <v>0</v>
       </c>
       <c r="F18">
-        <v>1.62290249796904</v>
+        <v>1.549828320424181</v>
       </c>
       <c r="G18">
         <v>0</v>
       </c>
       <c r="H18">
-        <v>0.5236828282628889</v>
+        <v>0.5147706092489056</v>
       </c>
       <c r="I18">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="19" spans="1:9">
@@ -1390,10 +1390,10 @@
         <v>0</v>
       </c>
       <c r="H19">
-        <v>0.6193974201557383</v>
+        <v>0.6099090717422234</v>
       </c>
       <c r="I19">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="20" spans="1:9">
@@ -1419,10 +1419,10 @@
         <v>0</v>
       </c>
       <c r="H20">
-        <v>0.4875660045010098</v>
+        <v>0.4863016023223692</v>
       </c>
       <c r="I20">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="21" spans="1:9">
@@ -1448,10 +1448,10 @@
         <v>0</v>
       </c>
       <c r="H21">
-        <v>0.4875660045010098</v>
+        <v>0.4863016023223692</v>
       </c>
       <c r="I21">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="22" spans="1:9">
@@ -1477,10 +1477,10 @@
         <v>0</v>
       </c>
       <c r="H22">
-        <v>0.5781396320332904</v>
+        <v>0.5760086226813654</v>
       </c>
       <c r="I22">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="23" spans="1:9">
@@ -1506,10 +1506,10 @@
         <v>0</v>
       </c>
       <c r="H23">
-        <v>0.4875660045010098</v>
+        <v>0.4863016023223692</v>
       </c>
       <c r="I23">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="24" spans="1:9">
@@ -1535,10 +1535,10 @@
         <v>0</v>
       </c>
       <c r="H24">
-        <v>0.4875660045010098</v>
+        <v>0.4863016023223692</v>
       </c>
       <c r="I24">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="25" spans="1:9">
@@ -1558,16 +1558,16 @@
         <v>0</v>
       </c>
       <c r="F25">
-        <v>0.5589989523206498</v>
+        <v>0.530839023295139</v>
       </c>
       <c r="G25">
         <v>0</v>
       </c>
       <c r="H25">
-        <v>0.5781396320332904</v>
+        <v>0.5760086226813654</v>
       </c>
       <c r="I25">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="26" spans="1:9">
@@ -1593,10 +1593,10 @@
         <v>0</v>
       </c>
       <c r="H26">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I26">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="27" spans="1:9">
@@ -1607,7 +1607,7 @@
         <v>12</v>
       </c>
       <c r="C27" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="D27">
         <v>0</v>
@@ -1622,10 +1622,10 @@
         <v>0</v>
       </c>
       <c r="H27">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I27">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="28" spans="1:9">
@@ -1651,10 +1651,10 @@
         <v>0</v>
       </c>
       <c r="H28">
-        <v>0.6038451386425255</v>
+        <v>0.5899789573712763</v>
       </c>
       <c r="I28">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="29" spans="1:9">
@@ -1680,10 +1680,10 @@
         <v>0</v>
       </c>
       <c r="H29">
-        <v>0.5121753915281123</v>
+        <v>0.5034589633872408</v>
       </c>
       <c r="I29">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="30" spans="1:9">
@@ -1709,10 +1709,10 @@
         <v>0</v>
       </c>
       <c r="H30">
-        <v>0.5121753915281123</v>
+        <v>0.5034589633872408</v>
       </c>
       <c r="I30">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="31" spans="1:9">
@@ -1738,10 +1738,10 @@
         <v>0</v>
       </c>
       <c r="H31">
-        <v>0.6071322078439527</v>
+        <v>0.5969001189112392</v>
       </c>
       <c r="I31">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="32" spans="1:9">
@@ -1767,10 +1767,10 @@
         <v>0</v>
       </c>
       <c r="H32">
-        <v>0.5236828282628889</v>
+        <v>0.5147706092489056</v>
       </c>
       <c r="I32">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="33" spans="1:9">
@@ -1796,10 +1796,10 @@
         <v>0</v>
       </c>
       <c r="H33">
-        <v>0.5236828282628889</v>
+        <v>0.5147706092489056</v>
       </c>
       <c r="I33">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="34" spans="1:9">
@@ -1819,16 +1819,16 @@
         <v>0</v>
       </c>
       <c r="F34">
-        <v>1.248459659689971</v>
+        <v>1.18556770745619</v>
       </c>
       <c r="G34">
         <v>0</v>
       </c>
       <c r="H34">
-        <v>0.6233123679910603</v>
+        <v>0.6128077276270587</v>
       </c>
       <c r="I34">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="35" spans="1:9">
@@ -1854,10 +1854,10 @@
         <v>0</v>
       </c>
       <c r="H35">
-        <v>0.4875660045010098</v>
+        <v>0.4863016023223692</v>
       </c>
       <c r="I35">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="36" spans="1:9">
@@ -1883,10 +1883,10 @@
         <v>0</v>
       </c>
       <c r="H36">
-        <v>0.4875660045010098</v>
+        <v>0.4863016023223692</v>
       </c>
       <c r="I36">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="37" spans="1:9">
@@ -1912,10 +1912,10 @@
         <v>0</v>
       </c>
       <c r="H37">
-        <v>0.5781396320332904</v>
+        <v>0.5760086226813654</v>
       </c>
       <c r="I37">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="38" spans="1:9">
@@ -1941,10 +1941,10 @@
         <v>0</v>
       </c>
       <c r="H38">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I38">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="39" spans="1:9">
@@ -1970,10 +1970,10 @@
         <v>0</v>
       </c>
       <c r="H39">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I39">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="40" spans="1:9">
@@ -1993,16 +1993,16 @@
         <v>0</v>
       </c>
       <c r="F40">
-        <v>0.5589989523206498</v>
+        <v>0.530839023295139</v>
       </c>
       <c r="G40">
         <v>0</v>
       </c>
       <c r="H40">
-        <v>0.607661787116463</v>
+        <v>0.592782893328202</v>
       </c>
       <c r="I40">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="41" spans="1:9">
@@ -2013,7 +2013,7 @@
         <v>10</v>
       </c>
       <c r="C41" t="s">
-        <v>42</v>
+        <v>11</v>
       </c>
       <c r="D41">
         <v>0</v>
@@ -2028,10 +2028,10 @@
         <v>0</v>
       </c>
       <c r="H41">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I41">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="42" spans="1:9">
@@ -2057,15 +2057,15 @@
         <v>0</v>
       </c>
       <c r="H42">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I42">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="43" spans="1:9">
       <c r="A43" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B43" t="s">
         <v>14</v>
@@ -2086,15 +2086,15 @@
         <v>0</v>
       </c>
       <c r="H43">
-        <v>0.6038451386425255</v>
+        <v>0.5899789573712763</v>
       </c>
       <c r="I43">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="44" spans="1:9">
       <c r="A44" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B44" t="s">
         <v>10</v>
@@ -2115,15 +2115,15 @@
         <v>0</v>
       </c>
       <c r="H44">
-        <v>0.5121753915281123</v>
+        <v>0.5034589633872408</v>
       </c>
       <c r="I44">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="45" spans="1:9">
       <c r="A45" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B45" t="s">
         <v>12</v>
@@ -2144,15 +2144,15 @@
         <v>0</v>
       </c>
       <c r="H45">
-        <v>0.5121753915281123</v>
+        <v>0.5034589633872408</v>
       </c>
       <c r="I45">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="46" spans="1:9">
       <c r="A46" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B46" t="s">
         <v>14</v>
@@ -2173,15 +2173,15 @@
         <v>0</v>
       </c>
       <c r="H46">
-        <v>0.6071322078439527</v>
+        <v>0.5969001189112392</v>
       </c>
       <c r="I46">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="47" spans="1:9">
       <c r="A47" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B47" t="s">
         <v>10</v>
@@ -2202,15 +2202,15 @@
         <v>0</v>
       </c>
       <c r="H47">
-        <v>0.5236828282628889</v>
+        <v>0.5147706092489056</v>
       </c>
       <c r="I47">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="48" spans="1:9">
       <c r="A48" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B48" t="s">
         <v>12</v>
@@ -2231,15 +2231,15 @@
         <v>0</v>
       </c>
       <c r="H48">
-        <v>0.5236828282628889</v>
+        <v>0.5147706092489056</v>
       </c>
       <c r="I48">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="49" spans="1:9">
       <c r="A49" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B49" t="s">
         <v>14</v>
@@ -2260,15 +2260,15 @@
         <v>0</v>
       </c>
       <c r="H49">
-        <v>0.6233123679910603</v>
+        <v>0.6128077276270587</v>
       </c>
       <c r="I49">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="50" spans="1:9">
       <c r="A50" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B50" t="s">
         <v>10</v>
@@ -2289,21 +2289,21 @@
         <v>0</v>
       </c>
       <c r="H50">
-        <v>0.4875660045010098</v>
+        <v>0.4863016023223692</v>
       </c>
       <c r="I50">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="51" spans="1:9">
       <c r="A51" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B51" t="s">
         <v>12</v>
       </c>
       <c r="C51" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="D51">
         <v>0</v>
@@ -2318,10 +2318,10 @@
         <v>0</v>
       </c>
       <c r="H51">
-        <v>0.4875660045010098</v>
+        <v>0.4863016023223692</v>
       </c>
       <c r="I51">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="52" spans="1:9">
@@ -2332,7 +2332,7 @@
         <v>14</v>
       </c>
       <c r="C52" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="D52">
         <v>0</v>
@@ -2347,10 +2347,10 @@
         <v>0</v>
       </c>
       <c r="H52">
-        <v>0.5781396320332904</v>
+        <v>0.5760086226813654</v>
       </c>
       <c r="I52">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="53" spans="1:9">
@@ -2376,10 +2376,10 @@
         <v>0</v>
       </c>
       <c r="H53">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I53">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="54" spans="1:9">
@@ -2405,10 +2405,10 @@
         <v>0</v>
       </c>
       <c r="H54">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I54">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="55" spans="1:9">
@@ -2434,10 +2434,10 @@
         <v>0</v>
       </c>
       <c r="H55">
-        <v>0.607661787116463</v>
+        <v>0.592782893328202</v>
       </c>
       <c r="I55">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="56" spans="1:9">
@@ -2463,10 +2463,10 @@
         <v>0</v>
       </c>
       <c r="H56">
-        <v>0.4875660045010098</v>
+        <v>0.4863016023223692</v>
       </c>
       <c r="I56">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="57" spans="1:9">
@@ -2492,10 +2492,10 @@
         <v>0</v>
       </c>
       <c r="H57">
-        <v>0.4875660045010098</v>
+        <v>0.4863016023223692</v>
       </c>
       <c r="I57">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="58" spans="1:9">
@@ -2521,10 +2521,10 @@
         <v>0</v>
       </c>
       <c r="H58">
-        <v>0.5781396320332904</v>
+        <v>0.5760086226813654</v>
       </c>
       <c r="I58">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="59" spans="1:9">
@@ -2550,10 +2550,10 @@
         <v>0</v>
       </c>
       <c r="H59">
-        <v>0.5201794499521184</v>
+        <v>0.5079155264285911</v>
       </c>
       <c r="I59">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="60" spans="1:9">
@@ -2579,10 +2579,10 @@
         <v>0</v>
       </c>
       <c r="H60">
-        <v>0.5201794499521184</v>
+        <v>0.5079155264285911</v>
       </c>
       <c r="I60">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="61" spans="1:9">
@@ -2608,10 +2608,10 @@
         <v>0</v>
       </c>
       <c r="H61">
-        <v>0.6071322078439527</v>
+        <v>0.5969001189112392</v>
       </c>
       <c r="I61">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="62" spans="1:9">
@@ -2622,7 +2622,7 @@
         <v>10</v>
       </c>
       <c r="C62" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="D62">
         <v>0</v>
@@ -2631,16 +2631,16 @@
         <v>0</v>
       </c>
       <c r="F62">
-        <v>1.662103921251415</v>
+        <v>0</v>
       </c>
       <c r="G62">
         <v>0</v>
       </c>
       <c r="H62">
-        <v>0.5236828282628889</v>
+        <v>0.5147706092489056</v>
       </c>
       <c r="I62">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="63" spans="1:9">
@@ -2660,16 +2660,16 @@
         <v>0</v>
       </c>
       <c r="F63">
-        <v>1.662103921251415</v>
+        <v>0</v>
       </c>
       <c r="G63">
         <v>0</v>
       </c>
       <c r="H63">
-        <v>0.5236828282628889</v>
+        <v>0.5147706092489056</v>
       </c>
       <c r="I63">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="64" spans="1:9">
@@ -2680,7 +2680,7 @@
         <v>14</v>
       </c>
       <c r="C64" t="s">
-        <v>11</v>
+        <v>48</v>
       </c>
       <c r="D64">
         <v>0</v>
@@ -2689,16 +2689,16 @@
         <v>0</v>
       </c>
       <c r="F64">
-        <v>1.278616366967039</v>
+        <v>0</v>
       </c>
       <c r="G64">
         <v>0</v>
       </c>
       <c r="H64">
-        <v>0.6233123679910603</v>
+        <v>0.6128077276270587</v>
       </c>
       <c r="I64">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="65" spans="1:9">
@@ -2724,10 +2724,10 @@
         <v>0</v>
       </c>
       <c r="H65">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I65">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="66" spans="1:9">
@@ -2753,10 +2753,10 @@
         <v>0</v>
       </c>
       <c r="H66">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I66">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="67" spans="1:9">
@@ -2776,16 +2776,16 @@
         <v>0</v>
       </c>
       <c r="F67">
-        <v>0.6286102326057974</v>
+        <v>0.5969435909038734</v>
       </c>
       <c r="G67">
         <v>0</v>
       </c>
       <c r="H67">
-        <v>0.6038451386425255</v>
+        <v>0.5899789573712763</v>
       </c>
       <c r="I67">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="68" spans="1:9">
@@ -2805,16 +2805,16 @@
         <v>0</v>
       </c>
       <c r="F68">
-        <v>0.7266560749816646</v>
+        <v>0.6939370452779632</v>
       </c>
       <c r="G68">
         <v>0</v>
       </c>
       <c r="H68">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I68">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="69" spans="1:9">
@@ -2834,16 +2834,16 @@
         <v>0</v>
       </c>
       <c r="F69">
-        <v>0.7266560749816646</v>
+        <v>0.6939370452779632</v>
       </c>
       <c r="G69">
         <v>0</v>
       </c>
       <c r="H69">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I69">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="70" spans="1:9">
@@ -2863,16 +2863,16 @@
         <v>0</v>
       </c>
       <c r="F70">
-        <v>0.5589989523206498</v>
+        <v>0.530839023295139</v>
       </c>
       <c r="G70">
         <v>0</v>
       </c>
       <c r="H70">
-        <v>0.6038451386425255</v>
+        <v>0.5899789573712763</v>
       </c>
       <c r="I70">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="71" spans="1:9">
@@ -2898,10 +2898,10 @@
         <v>0</v>
       </c>
       <c r="H71">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I71">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="72" spans="1:9">
@@ -2927,10 +2927,10 @@
         <v>0</v>
       </c>
       <c r="H72">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I72">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="73" spans="1:9">
@@ -2956,10 +2956,10 @@
         <v>0</v>
       </c>
       <c r="H73">
-        <v>0.6038451386425255</v>
+        <v>0.5899789573712763</v>
       </c>
       <c r="I73">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="74" spans="1:9">
@@ -2985,10 +2985,10 @@
         <v>0</v>
       </c>
       <c r="H74">
-        <v>0.51097824370969</v>
+        <v>0.5130400073790439</v>
       </c>
       <c r="I74">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="75" spans="1:9">
@@ -3014,10 +3014,10 @@
         <v>0</v>
       </c>
       <c r="H75">
-        <v>0.51097824370969</v>
+        <v>0.5130400073790439</v>
       </c>
       <c r="I75">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="76" spans="1:9">
@@ -3043,10 +3043,10 @@
         <v>0</v>
       </c>
       <c r="H76">
-        <v>0.5916768885176681</v>
+        <v>0.594113883169007</v>
       </c>
       <c r="I76">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="77" spans="1:9">
@@ -3072,10 +3072,10 @@
         <v>0</v>
       </c>
       <c r="H77">
-        <v>0.4981527456827964</v>
+        <v>0.5001512095680933</v>
       </c>
       <c r="I77">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="78" spans="1:9">
@@ -3101,10 +3101,10 @@
         <v>0</v>
       </c>
       <c r="H78">
-        <v>0.4981527456827964</v>
+        <v>0.5001512095680933</v>
       </c>
       <c r="I78">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="79" spans="1:9">
@@ -3130,10 +3130,10 @@
         <v>0</v>
       </c>
       <c r="H79">
-        <v>0.5930298575827418</v>
+        <v>0.5954668043423548</v>
       </c>
       <c r="I79">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="80" spans="1:9">
@@ -3159,10 +3159,10 @@
         <v>0</v>
       </c>
       <c r="H80">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I80">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="81" spans="1:9">
@@ -3188,10 +3188,10 @@
         <v>0</v>
       </c>
       <c r="H81">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I81">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="82" spans="1:9">
@@ -3217,10 +3217,10 @@
         <v>0</v>
       </c>
       <c r="H82">
-        <v>0.6038451386425255</v>
+        <v>0.5899789573712763</v>
       </c>
       <c r="I82">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="83" spans="1:9">
@@ -3231,7 +3231,7 @@
         <v>10</v>
       </c>
       <c r="C83" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="D83">
         <v>0</v>
@@ -3246,10 +3246,10 @@
         <v>0</v>
       </c>
       <c r="H83">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I83">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="84" spans="1:9">
@@ -3275,10 +3275,10 @@
         <v>0</v>
       </c>
       <c r="H84">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I84">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="85" spans="1:9">
@@ -3301,13 +3301,13 @@
         <v>0</v>
       </c>
       <c r="G85">
-        <v>0.5589989523206498</v>
+        <v>0.530839023295139</v>
       </c>
       <c r="H85">
-        <v>0.6038451386425255</v>
+        <v>0.5899789573712763</v>
       </c>
       <c r="I85">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="86" spans="1:9">
@@ -3333,10 +3333,10 @@
         <v>0</v>
       </c>
       <c r="H86">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I86">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="87" spans="1:9">
@@ -3362,10 +3362,10 @@
         <v>0</v>
       </c>
       <c r="H87">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I87">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="88" spans="1:9">
@@ -3391,10 +3391,10 @@
         <v>0</v>
       </c>
       <c r="H88">
-        <v>0.6038451386425255</v>
+        <v>0.5899789573712763</v>
       </c>
       <c r="I88">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="89" spans="1:9">
@@ -3420,10 +3420,10 @@
         <v>0</v>
       </c>
       <c r="H89">
-        <v>0.5121753915281123</v>
+        <v>0.5034589633872408</v>
       </c>
       <c r="I89">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="90" spans="1:9">
@@ -3449,10 +3449,10 @@
         <v>0</v>
       </c>
       <c r="H90">
-        <v>0.5121753915281123</v>
+        <v>0.5034589633872408</v>
       </c>
       <c r="I90">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="91" spans="1:9">
@@ -3478,10 +3478,10 @@
         <v>0</v>
       </c>
       <c r="H91">
-        <v>0.6033188855918793</v>
+        <v>0.5940767079711704</v>
       </c>
       <c r="I91">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="92" spans="1:9">
@@ -3507,10 +3507,10 @@
         <v>0</v>
       </c>
       <c r="H92">
-        <v>0.5236828282628889</v>
+        <v>0.5147706092489056</v>
       </c>
       <c r="I92">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="93" spans="1:9">
@@ -3536,10 +3536,10 @@
         <v>0</v>
       </c>
       <c r="H93">
-        <v>0.5236828282628889</v>
+        <v>0.5147706092489056</v>
       </c>
       <c r="I93">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="94" spans="1:9">
@@ -3559,16 +3559,16 @@
         <v>0</v>
       </c>
       <c r="F94">
-        <v>1.248459659689971</v>
+        <v>1.18556770745619</v>
       </c>
       <c r="G94">
         <v>0</v>
       </c>
       <c r="H94">
-        <v>0.6233123679910603</v>
+        <v>0.6128077276270587</v>
       </c>
       <c r="I94">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="95" spans="1:9">
@@ -3594,10 +3594,10 @@
         <v>0</v>
       </c>
       <c r="H95">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I95">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="96" spans="1:9">
@@ -3623,10 +3623,10 @@
         <v>0</v>
       </c>
       <c r="H96">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I96">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="97" spans="1:9">
@@ -3652,10 +3652,10 @@
         <v>0</v>
       </c>
       <c r="H97">
-        <v>0.607661787116463</v>
+        <v>0.592782893328202</v>
       </c>
       <c r="I97">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="98" spans="1:9">
@@ -3681,10 +3681,10 @@
         <v>0</v>
       </c>
       <c r="H98">
-        <v>0.4875660045010098</v>
+        <v>0.4863016023223692</v>
       </c>
       <c r="I98">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="99" spans="1:9">
@@ -3710,10 +3710,10 @@
         <v>0</v>
       </c>
       <c r="H99">
-        <v>0.4875660045010098</v>
+        <v>0.4863016023223692</v>
       </c>
       <c r="I99">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="100" spans="1:9">
@@ -3733,16 +3733,16 @@
         <v>0</v>
       </c>
       <c r="F100">
-        <v>0.5589989523206498</v>
+        <v>0.530839023295139</v>
       </c>
       <c r="G100">
         <v>0</v>
       </c>
       <c r="H100">
-        <v>0.5781396320332904</v>
+        <v>0.5760086226813654</v>
       </c>
       <c r="I100">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="101" spans="1:9">
@@ -3768,10 +3768,10 @@
         <v>0</v>
       </c>
       <c r="H101">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I101">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="102" spans="1:9">
@@ -3782,7 +3782,7 @@
         <v>12</v>
       </c>
       <c r="C102" t="s">
-        <v>42</v>
+        <v>11</v>
       </c>
       <c r="D102">
         <v>0</v>
@@ -3797,10 +3797,10 @@
         <v>0</v>
       </c>
       <c r="H102">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I102">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="103" spans="1:9">
@@ -3826,10 +3826,10 @@
         <v>0</v>
       </c>
       <c r="H103">
-        <v>0.607661787116463</v>
+        <v>0.592782893328202</v>
       </c>
       <c r="I103">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="104" spans="1:9">
@@ -3855,10 +3855,10 @@
         <v>0</v>
       </c>
       <c r="H104">
-        <v>0.5121753915281123</v>
+        <v>0.5034589633872408</v>
       </c>
       <c r="I104">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="105" spans="1:9">
@@ -3884,10 +3884,10 @@
         <v>0</v>
       </c>
       <c r="H105">
-        <v>0.5121753915281123</v>
+        <v>0.5034589633872408</v>
       </c>
       <c r="I105">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="106" spans="1:9">
@@ -3907,16 +3907,16 @@
         <v>0</v>
       </c>
       <c r="F106">
-        <v>6.103580558484303</v>
+        <v>5.796108792008049</v>
       </c>
       <c r="G106">
         <v>0</v>
       </c>
       <c r="H106">
-        <v>0.6071322078439527</v>
+        <v>0.5969001189112392</v>
       </c>
       <c r="I106">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="107" spans="1:9">
@@ -3942,10 +3942,10 @@
         <v>0</v>
       </c>
       <c r="H107">
-        <v>0.5236828282628889</v>
+        <v>0.5147706092489056</v>
       </c>
       <c r="I107">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="108" spans="1:9">
@@ -3971,10 +3971,10 @@
         <v>0</v>
       </c>
       <c r="H108">
-        <v>0.5236828282628889</v>
+        <v>0.5147706092489056</v>
       </c>
       <c r="I108">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="109" spans="1:9">
@@ -4000,10 +4000,10 @@
         <v>0</v>
       </c>
       <c r="H109">
-        <v>0.6233123679910603</v>
+        <v>0.6128077276270587</v>
       </c>
       <c r="I109">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="110" spans="1:9">
@@ -4014,7 +4014,7 @@
         <v>10</v>
       </c>
       <c r="C110" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="D110">
         <v>0</v>
@@ -4029,10 +4029,10 @@
         <v>0</v>
       </c>
       <c r="H110">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I110">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="111" spans="1:9">
@@ -4058,10 +4058,10 @@
         <v>0</v>
       </c>
       <c r="H111">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I111">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="112" spans="1:9">
@@ -4087,10 +4087,10 @@
         <v>0</v>
       </c>
       <c r="H112">
-        <v>0.607661787116463</v>
+        <v>0.592782893328202</v>
       </c>
       <c r="I112">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="113" spans="1:9">
@@ -4116,10 +4116,10 @@
         <v>0</v>
       </c>
       <c r="H113">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I113">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="114" spans="1:9">
@@ -4145,10 +4145,10 @@
         <v>0</v>
       </c>
       <c r="H114">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I114">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="115" spans="1:9">
@@ -4171,13 +4171,13 @@
         <v>0</v>
       </c>
       <c r="G115">
-        <v>0.5589989523206498</v>
+        <v>0.530839023295139</v>
       </c>
       <c r="H115">
-        <v>0.6038451386425255</v>
+        <v>0.5899789573712763</v>
       </c>
       <c r="I115">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="116" spans="1:9">
@@ -4203,10 +4203,10 @@
         <v>0</v>
       </c>
       <c r="H116">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I116">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="117" spans="1:9">
@@ -4232,10 +4232,10 @@
         <v>0</v>
       </c>
       <c r="H117">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I117">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="118" spans="1:9">
@@ -4261,10 +4261,10 @@
         <v>0</v>
       </c>
       <c r="H118">
-        <v>0.607661787116463</v>
+        <v>0.592782893328202</v>
       </c>
       <c r="I118">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="119" spans="1:9">
@@ -4290,10 +4290,10 @@
         <v>0</v>
       </c>
       <c r="H119">
-        <v>0.4872063084581594</v>
+        <v>0.4891608125674324</v>
       </c>
       <c r="I119">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="120" spans="1:9">
@@ -4319,10 +4319,10 @@
         <v>0</v>
       </c>
       <c r="H120">
-        <v>0.4872063084581594</v>
+        <v>0.4891608125674324</v>
       </c>
       <c r="I120">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="121" spans="1:9">
@@ -4348,10 +4348,10 @@
         <v>0</v>
       </c>
       <c r="H121">
-        <v>0.577635781417318</v>
+        <v>0.5800093410962281</v>
       </c>
       <c r="I121">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="122" spans="1:9">
@@ -4377,10 +4377,10 @@
         <v>0</v>
       </c>
       <c r="H122">
-        <v>0.5236828282628889</v>
+        <v>0.5147706092489056</v>
       </c>
       <c r="I122">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="123" spans="1:9">
@@ -4406,10 +4406,10 @@
         <v>0</v>
       </c>
       <c r="H123">
-        <v>0.5236828282628889</v>
+        <v>0.5147706092489056</v>
       </c>
       <c r="I123">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="124" spans="1:9">
@@ -4435,10 +4435,10 @@
         <v>0</v>
       </c>
       <c r="H124">
-        <v>0.6233123679910603</v>
+        <v>0.6128077276270587</v>
       </c>
       <c r="I124">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="125" spans="1:9">
@@ -4464,10 +4464,10 @@
         <v>0</v>
       </c>
       <c r="H125">
-        <v>0.4875660045010098</v>
+        <v>0.4863016023223692</v>
       </c>
       <c r="I125">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="126" spans="1:9">
@@ -4478,7 +4478,7 @@
         <v>12</v>
       </c>
       <c r="C126" t="s">
-        <v>42</v>
+        <v>15</v>
       </c>
       <c r="D126">
         <v>0</v>
@@ -4493,10 +4493,10 @@
         <v>0</v>
       </c>
       <c r="H126">
-        <v>0.4875660045010098</v>
+        <v>0.4863016023223692</v>
       </c>
       <c r="I126">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="127" spans="1:9">
@@ -4507,7 +4507,7 @@
         <v>14</v>
       </c>
       <c r="C127" t="s">
-        <v>42</v>
+        <v>11</v>
       </c>
       <c r="D127">
         <v>0</v>
@@ -4522,10 +4522,10 @@
         <v>0</v>
       </c>
       <c r="H127">
-        <v>0.5781396320332904</v>
+        <v>0.5760086226813654</v>
       </c>
       <c r="I127">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="128" spans="1:9">
@@ -4551,10 +4551,10 @@
         <v>0</v>
       </c>
       <c r="H128">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I128">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="129" spans="1:9">
@@ -4580,10 +4580,10 @@
         <v>0</v>
       </c>
       <c r="H129">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I129">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="130" spans="1:9">
@@ -4609,10 +4609,10 @@
         <v>0</v>
       </c>
       <c r="H130">
-        <v>0.607661787116463</v>
+        <v>0.592782893328202</v>
       </c>
       <c r="I130">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="131" spans="1:9">
@@ -4623,7 +4623,7 @@
         <v>10</v>
       </c>
       <c r="C131" t="s">
-        <v>42</v>
+        <v>11</v>
       </c>
       <c r="D131">
         <v>0</v>
@@ -4638,10 +4638,10 @@
         <v>0</v>
       </c>
       <c r="H131">
-        <v>0.4875660045010098</v>
+        <v>0.4863016023223692</v>
       </c>
       <c r="I131">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="132" spans="1:9">
@@ -4652,7 +4652,7 @@
         <v>12</v>
       </c>
       <c r="C132" t="s">
-        <v>42</v>
+        <v>11</v>
       </c>
       <c r="D132">
         <v>0</v>
@@ -4667,10 +4667,10 @@
         <v>0</v>
       </c>
       <c r="H132">
-        <v>0.4875660045010098</v>
+        <v>0.4863016023223692</v>
       </c>
       <c r="I132">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="133" spans="1:9">
@@ -4696,10 +4696,10 @@
         <v>0</v>
       </c>
       <c r="H133">
-        <v>0.5781396320332904</v>
+        <v>0.5760086226813654</v>
       </c>
       <c r="I133">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="134" spans="1:9">
@@ -4725,10 +4725,10 @@
         <v>0</v>
       </c>
       <c r="H134">
-        <v>0.5201794499521184</v>
+        <v>0.5079155264285911</v>
       </c>
       <c r="I134">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="135" spans="1:9">
@@ -4754,10 +4754,10 @@
         <v>0</v>
       </c>
       <c r="H135">
-        <v>0.5201794499521184</v>
+        <v>0.5079155264285911</v>
       </c>
       <c r="I135">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="136" spans="1:9">
@@ -4783,10 +4783,10 @@
         <v>0</v>
       </c>
       <c r="H136">
-        <v>0.6071322078439527</v>
+        <v>0.5969001189112392</v>
       </c>
       <c r="I136">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="137" spans="1:9">
@@ -4812,10 +4812,10 @@
         <v>0</v>
       </c>
       <c r="H137">
-        <v>0.4981527456827964</v>
+        <v>0.5001512095680933</v>
       </c>
       <c r="I137">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="138" spans="1:9">
@@ -4841,10 +4841,10 @@
         <v>0</v>
       </c>
       <c r="H138">
-        <v>0.4981527456827964</v>
+        <v>0.5001512095680933</v>
       </c>
       <c r="I138">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="139" spans="1:9">
@@ -4870,10 +4870,10 @@
         <v>0</v>
       </c>
       <c r="H139">
-        <v>0.5930298575827418</v>
+        <v>0.5954668043423548</v>
       </c>
       <c r="I139">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="140" spans="1:9">
@@ -4899,10 +4899,10 @@
         <v>0</v>
       </c>
       <c r="H140">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I140">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="141" spans="1:9">
@@ -4928,10 +4928,10 @@
         <v>0</v>
       </c>
       <c r="H141">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I141">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="142" spans="1:9">
@@ -4957,10 +4957,10 @@
         <v>0</v>
       </c>
       <c r="H142">
-        <v>0.6038451386425255</v>
+        <v>0.5899789573712763</v>
       </c>
       <c r="I142">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="143" spans="1:9">
@@ -4980,16 +4980,16 @@
         <v>0</v>
       </c>
       <c r="F143">
-        <v>0.7266560749816646</v>
+        <v>0.6939370452779632</v>
       </c>
       <c r="G143">
         <v>0</v>
       </c>
       <c r="H143">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I143">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="144" spans="1:9">
@@ -5009,16 +5009,16 @@
         <v>0</v>
       </c>
       <c r="F144">
-        <v>0.7266560749816646</v>
+        <v>0.6939370452779632</v>
       </c>
       <c r="G144">
         <v>0</v>
       </c>
       <c r="H144">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I144">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="145" spans="1:9">
@@ -5038,16 +5038,16 @@
         <v>0</v>
       </c>
       <c r="F145">
-        <v>0.5589989523206498</v>
+        <v>0.530839023295139</v>
       </c>
       <c r="G145">
         <v>0</v>
       </c>
       <c r="H145">
-        <v>0.6038451386425255</v>
+        <v>0.5899789573712763</v>
       </c>
       <c r="I145">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="146" spans="1:9">
@@ -5073,10 +5073,10 @@
         <v>0</v>
       </c>
       <c r="H146">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I146">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="147" spans="1:9">
@@ -5102,10 +5102,10 @@
         <v>0</v>
       </c>
       <c r="H147">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I147">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="148" spans="1:9">
@@ -5131,10 +5131,10 @@
         <v>0</v>
       </c>
       <c r="H148">
-        <v>0.6038451386425255</v>
+        <v>0.5899789573712763</v>
       </c>
       <c r="I148">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="149" spans="1:9">
@@ -5160,10 +5160,10 @@
         <v>0</v>
       </c>
       <c r="H149">
-        <v>0.5121753915281123</v>
+        <v>0.5130400073790439</v>
       </c>
       <c r="I149">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="150" spans="1:9">
@@ -5189,10 +5189,10 @@
         <v>0</v>
       </c>
       <c r="H150">
-        <v>0.5121753915281123</v>
+        <v>0.5130400073790439</v>
       </c>
       <c r="I150">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="151" spans="1:9">
@@ -5218,10 +5218,10 @@
         <v>0</v>
       </c>
       <c r="H151">
-        <v>0.6033188855918793</v>
+        <v>0.594113883169007</v>
       </c>
       <c r="I151">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="152" spans="1:9">
@@ -5247,10 +5247,10 @@
         <v>0</v>
       </c>
       <c r="H152">
-        <v>0.5236828282628889</v>
+        <v>0.5147706092489056</v>
       </c>
       <c r="I152">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="153" spans="1:9">
@@ -5276,10 +5276,10 @@
         <v>0</v>
       </c>
       <c r="H153">
-        <v>0.5236828282628889</v>
+        <v>0.5147706092489056</v>
       </c>
       <c r="I153">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="154" spans="1:9">
@@ -5305,10 +5305,10 @@
         <v>0</v>
       </c>
       <c r="H154">
-        <v>0.6233123679910603</v>
+        <v>0.6128077276270587</v>
       </c>
       <c r="I154">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="155" spans="1:9">
@@ -5334,10 +5334,10 @@
         <v>0</v>
       </c>
       <c r="H155">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I155">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="156" spans="1:9">
@@ -5363,10 +5363,10 @@
         <v>0</v>
       </c>
       <c r="H156">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I156">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="157" spans="1:9">
@@ -5377,7 +5377,7 @@
         <v>14</v>
       </c>
       <c r="C157" t="s">
-        <v>42</v>
+        <v>15</v>
       </c>
       <c r="D157">
         <v>0</v>
@@ -5392,10 +5392,10 @@
         <v>0</v>
       </c>
       <c r="H157">
-        <v>0.607661787116463</v>
+        <v>0.592782893328202</v>
       </c>
       <c r="I157">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="158" spans="1:9">
@@ -5421,10 +5421,10 @@
         <v>0</v>
       </c>
       <c r="H158">
-        <v>0.4875660045010098</v>
+        <v>0.4863016023223692</v>
       </c>
       <c r="I158">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="159" spans="1:9">
@@ -5450,10 +5450,10 @@
         <v>0</v>
       </c>
       <c r="H159">
-        <v>0.4875660045010098</v>
+        <v>0.4863016023223692</v>
       </c>
       <c r="I159">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="160" spans="1:9">
@@ -5479,10 +5479,10 @@
         <v>0</v>
       </c>
       <c r="H160">
-        <v>0.5781396320332904</v>
+        <v>0.5760086226813654</v>
       </c>
       <c r="I160">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="161" spans="1:9">
@@ -5493,7 +5493,7 @@
         <v>10</v>
       </c>
       <c r="C161" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="D161">
         <v>0</v>
@@ -5508,10 +5508,10 @@
         <v>0</v>
       </c>
       <c r="H161">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I161">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="162" spans="1:9">
@@ -5522,7 +5522,7 @@
         <v>12</v>
       </c>
       <c r="C162" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="D162">
         <v>0</v>
@@ -5537,10 +5537,10 @@
         <v>0</v>
       </c>
       <c r="H162">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I162">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="163" spans="1:9">
@@ -5551,7 +5551,7 @@
         <v>14</v>
       </c>
       <c r="C163" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="D163">
         <v>0</v>
@@ -5566,10 +5566,10 @@
         <v>0</v>
       </c>
       <c r="H163">
-        <v>0.607661787116463</v>
+        <v>0.592782893328202</v>
       </c>
       <c r="I163">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="164" spans="1:9">
@@ -5595,10 +5595,10 @@
         <v>0</v>
       </c>
       <c r="H164">
-        <v>0.5121753915281123</v>
+        <v>0.5034589633872408</v>
       </c>
       <c r="I164">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="165" spans="1:9">
@@ -5624,10 +5624,10 @@
         <v>0</v>
       </c>
       <c r="H165">
-        <v>0.5121753915281123</v>
+        <v>0.5034589633872408</v>
       </c>
       <c r="I165">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="166" spans="1:9">
@@ -5653,10 +5653,10 @@
         <v>0</v>
       </c>
       <c r="H166">
-        <v>0.6071322078439527</v>
+        <v>0.5969001189112392</v>
       </c>
       <c r="I166">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="167" spans="1:9">
@@ -5682,10 +5682,10 @@
         <v>0</v>
       </c>
       <c r="H167">
-        <v>0.5236828282628889</v>
+        <v>0.5147706092489056</v>
       </c>
       <c r="I167">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="168" spans="1:9">
@@ -5711,10 +5711,10 @@
         <v>0</v>
       </c>
       <c r="H168">
-        <v>0.5236828282628889</v>
+        <v>0.5147706092489056</v>
       </c>
       <c r="I168">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="169" spans="1:9">
@@ -5734,16 +5734,16 @@
         <v>0</v>
       </c>
       <c r="F169">
-        <v>1.248459659689971</v>
+        <v>1.18556770745619</v>
       </c>
       <c r="G169">
         <v>0</v>
       </c>
       <c r="H169">
-        <v>0.6233123679910603</v>
+        <v>0.6128077276270587</v>
       </c>
       <c r="I169">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="170" spans="1:9">
@@ -5769,10 +5769,10 @@
         <v>0</v>
       </c>
       <c r="H170">
-        <v>0.4875660045010098</v>
+        <v>0.4863016023223692</v>
       </c>
       <c r="I170">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="171" spans="1:9">
@@ -5798,10 +5798,10 @@
         <v>0</v>
       </c>
       <c r="H171">
-        <v>0.4875660045010098</v>
+        <v>0.4863016023223692</v>
       </c>
       <c r="I171">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="172" spans="1:9">
@@ -5827,10 +5827,10 @@
         <v>0</v>
       </c>
       <c r="H172">
-        <v>0.5781396320332904</v>
+        <v>0.5760086226813654</v>
       </c>
       <c r="I172">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="173" spans="1:9">
@@ -5850,16 +5850,16 @@
         <v>0</v>
       </c>
       <c r="F173">
-        <v>0.7266560749816646</v>
+        <v>0.6939370452779632</v>
       </c>
       <c r="G173">
         <v>0</v>
       </c>
       <c r="H173">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I173">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="174" spans="1:9">
@@ -5879,16 +5879,16 @@
         <v>0</v>
       </c>
       <c r="F174">
-        <v>0.7266560749816646</v>
+        <v>0.6939370452779632</v>
       </c>
       <c r="G174">
         <v>0</v>
       </c>
       <c r="H174">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I174">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="175" spans="1:9">
@@ -5908,16 +5908,16 @@
         <v>0</v>
       </c>
       <c r="F175">
-        <v>0.5589989523206498</v>
+        <v>0.530839023295139</v>
       </c>
       <c r="G175">
         <v>0</v>
       </c>
       <c r="H175">
-        <v>0.607661787116463</v>
+        <v>0.592782893328202</v>
       </c>
       <c r="I175">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="176" spans="1:9">
@@ -5943,10 +5943,10 @@
         <v>0</v>
       </c>
       <c r="H176">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I176">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="177" spans="1:9">
@@ -5972,10 +5972,10 @@
         <v>0</v>
       </c>
       <c r="H177">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I177">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="178" spans="1:9">
@@ -6001,10 +6001,10 @@
         <v>0</v>
       </c>
       <c r="H178">
-        <v>0.6038451386425255</v>
+        <v>0.5899789573712763</v>
       </c>
       <c r="I178">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="179" spans="1:9">
@@ -6030,10 +6030,10 @@
         <v>0</v>
       </c>
       <c r="H179">
-        <v>0.4872063084581594</v>
+        <v>0.4891608125674324</v>
       </c>
       <c r="I179">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="180" spans="1:9">
@@ -6059,10 +6059,10 @@
         <v>0</v>
       </c>
       <c r="H180">
-        <v>0.4872063084581594</v>
+        <v>0.4891608125674324</v>
       </c>
       <c r="I180">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="181" spans="1:9">
@@ -6088,10 +6088,10 @@
         <v>0</v>
       </c>
       <c r="H181">
-        <v>0.577635781417318</v>
+        <v>0.5800093410962281</v>
       </c>
       <c r="I181">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="182" spans="1:9">
@@ -6117,10 +6117,10 @@
         <v>0</v>
       </c>
       <c r="H182">
-        <v>0.5236828282628889</v>
+        <v>0.5147706092489056</v>
       </c>
       <c r="I182">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="183" spans="1:9">
@@ -6146,10 +6146,10 @@
         <v>0</v>
       </c>
       <c r="H183">
-        <v>0.5236828282628889</v>
+        <v>0.5147706092489056</v>
       </c>
       <c r="I183">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="184" spans="1:9">
@@ -6169,16 +6169,16 @@
         <v>0</v>
       </c>
       <c r="F184">
-        <v>1.248459659689971</v>
+        <v>1.18556770745619</v>
       </c>
       <c r="G184">
         <v>0</v>
       </c>
       <c r="H184">
-        <v>0.6233123679910603</v>
+        <v>0.6128077276270587</v>
       </c>
       <c r="I184">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="185" spans="1:9">
@@ -6204,10 +6204,10 @@
         <v>0</v>
       </c>
       <c r="H185">
-        <v>0.4875660045010098</v>
+        <v>0.4863016023223692</v>
       </c>
       <c r="I185">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="186" spans="1:9">
@@ -6233,10 +6233,10 @@
         <v>0</v>
       </c>
       <c r="H186">
-        <v>0.4875660045010098</v>
+        <v>0.4863016023223692</v>
       </c>
       <c r="I186">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="187" spans="1:9">
@@ -6262,10 +6262,10 @@
         <v>0</v>
       </c>
       <c r="H187">
-        <v>0.5781396320332904</v>
+        <v>0.5760086226813654</v>
       </c>
       <c r="I187">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="188" spans="1:9">
@@ -6285,16 +6285,16 @@
         <v>0</v>
       </c>
       <c r="F188">
-        <v>0.7266560749816646</v>
+        <v>0.6939370452779632</v>
       </c>
       <c r="G188">
         <v>0</v>
       </c>
       <c r="H188">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I188">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="189" spans="1:9">
@@ -6314,16 +6314,16 @@
         <v>0</v>
       </c>
       <c r="F189">
-        <v>0.7266560749816646</v>
+        <v>0.6939370452779632</v>
       </c>
       <c r="G189">
         <v>0</v>
       </c>
       <c r="H189">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I189">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="190" spans="1:9">
@@ -6346,13 +6346,13 @@
         <v>0</v>
       </c>
       <c r="G190">
-        <v>0.5589989523206498</v>
+        <v>0.530839023295139</v>
       </c>
       <c r="H190">
-        <v>0.6038451386425255</v>
+        <v>0.5899789573712763</v>
       </c>
       <c r="I190">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="191" spans="1:9">
@@ -6378,10 +6378,10 @@
         <v>0</v>
       </c>
       <c r="H191">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I191">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="192" spans="1:9">
@@ -6407,10 +6407,10 @@
         <v>0</v>
       </c>
       <c r="H192">
-        <v>0.5125535218157947</v>
+        <v>0.500516178542048</v>
       </c>
       <c r="I192">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="193" spans="1:9">
@@ -6430,16 +6430,16 @@
         <v>0</v>
       </c>
       <c r="F193">
-        <v>0.7115653566508024</v>
+        <v>0.6757197976258453</v>
       </c>
       <c r="G193">
         <v>0</v>
       </c>
       <c r="H193">
-        <v>0.6038451386425255</v>
+        <v>0.5899789573712763</v>
       </c>
       <c r="I193">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="194" spans="1:9">
@@ -6465,10 +6465,10 @@
         <v>0</v>
       </c>
       <c r="H194">
-        <v>0.5121753915281123</v>
+        <v>0.5034589633872408</v>
       </c>
       <c r="I194">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="195" spans="1:9">
@@ -6494,10 +6494,10 @@
         <v>0</v>
       </c>
       <c r="H195">
-        <v>0.5121753915281123</v>
+        <v>0.5034589633872408</v>
       </c>
       <c r="I195">
-        <v>0.1328468903598754</v>
+        <v>0.1277439555826503</v>
       </c>
     </row>
     <row r="196" spans="1:9">
@@ -6523,10 +6523,10 @@
         <v>0</v>
       </c>
       <c r="H196">
-        <v>0.6033188855918793</v>
+        <v>0.5940767079711704</v>
       </c>
       <c r="I196">
-        <v>0.1059297817849267</v>
+        <v>0.1012146274882231</v>
       </c>
     </row>
     <row r="197" spans="1:9">
@@ -6552,10 +6552,10 @@
         <v>0</v>
       </c>
       <c r="H197">
-        <v>0.5463198615344834</v>
+        <v>0.5485127775564219</v>
       </c>
       <c r="I197">
-        <v>0.1490265164416418</v>
+        <v>0.1425583099316179</v>
       </c>
     </row>
     <row r="198" spans="1:9">
@@ -6581,10 +6581,10 @@
         <v>0</v>
       </c>
       <c r="H198">
-        <v>0.5463198615344834</v>
+        <v>0.5485127775564219</v>
       </c>
       <c r="I198">
-        <v>0.1490265164416418</v>
+        <v>0.1425583099316179</v>
       </c>
     </row>
     <row r="199" spans="1:9">
@@ -6610,10 +6610,10 @@
         <v>0</v>
       </c>
       <c r="H199">
-        <v>0.5930298575827418</v>
+        <v>0.5954668043423548</v>
       </c>
       <c r="I199">
-        <v>0.1118728929202757</v>
+        <v>0.1065714798831008</v>
       </c>
     </row>
     <row r="200" spans="1:9">
@@ -6639,10 +6639,10 @@
         <v>0</v>
       </c>
       <c r="H200">
-        <v>0.5336129587278015</v>
+        <v>0.5318998173897364</v>
       </c>
       <c r="I200">
-        <v>0.1490265164416418</v>
+        <v>0.1425583099316179</v>
       </c>
     </row>
     <row r="201" spans="1:9">
@@ -6668,10 +6668,10 @@
         <v>0</v>
       </c>
       <c r="H201">
-        <v>0.5336129587278015</v>
+        <v>0.5318998173897364</v>
       </c>
       <c r="I201">
-        <v>0.1490265164416418</v>
+        <v>0.1425583099316179</v>
       </c>
     </row>
     <row r="202" spans="1:9">
@@ -6694,13 +6694,13 @@
         <v>0</v>
       </c>
       <c r="G202">
-        <v>0.6690851985516648</v>
+        <v>0.6329500884812544</v>
       </c>
       <c r="H202">
-        <v>0.5781396320332904</v>
+        <v>0.5760086226813654</v>
       </c>
       <c r="I202">
-        <v>0.1118728929202757</v>
+        <v>0.1065714798831008</v>
       </c>
     </row>
     <row r="203" spans="1:9">
@@ -6726,10 +6726,10 @@
         <v>0</v>
       </c>
       <c r="H203">
-        <v>0.5336129587278015</v>
+        <v>0.5318998173897364</v>
       </c>
       <c r="I203">
-        <v>0.1490265164416418</v>
+        <v>0.1425583099316179</v>
       </c>
     </row>
     <row r="204" spans="1:9">
@@ -6755,10 +6755,10 @@
         <v>0</v>
       </c>
       <c r="H204">
-        <v>0.5336129587278015</v>
+        <v>0.5318998173897364</v>
       </c>
       <c r="I204">
-        <v>0.1490265164416418</v>
+        <v>0.1425583099316179</v>
       </c>
     </row>
     <row r="205" spans="1:9">
@@ -6769,7 +6769,7 @@
         <v>14</v>
       </c>
       <c r="C205" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="D205">
         <v>0</v>
@@ -6778,16 +6778,16 @@
         <v>0</v>
       </c>
       <c r="F205">
-        <v>0.5949917860121468</v>
+        <v>0</v>
       </c>
       <c r="G205">
-        <v>0</v>
+        <v>0.5628582195768423</v>
       </c>
       <c r="H205">
-        <v>0.5781396320332904</v>
+        <v>0.5760086226813654</v>
       </c>
       <c r="I205">
-        <v>0.1118728929202757</v>
+        <v>0.1065714798831008</v>
       </c>
     </row>
     <row r="206" spans="1:9">
@@ -6798,7 +6798,7 @@
         <v>10</v>
       </c>
       <c r="C206" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="D206">
         <v>0</v>
@@ -6807,16 +6807,16 @@
         <v>0</v>
       </c>
       <c r="F206">
-        <v>1.06093561536766</v>
+        <v>0</v>
       </c>
       <c r="G206">
         <v>0</v>
       </c>
       <c r="H206">
-        <v>0.5609603597412309</v>
+        <v>0.5474472275965149</v>
       </c>
       <c r="I206">
-        <v>0.1490265164416418</v>
+        <v>0.1425583099316179</v>
       </c>
     </row>
     <row r="207" spans="1:9">
@@ -6827,7 +6827,7 @@
         <v>12</v>
       </c>
       <c r="C207" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="D207">
         <v>0</v>
@@ -6836,16 +6836,16 @@
         <v>0</v>
       </c>
       <c r="F207">
-        <v>1.06093561536766</v>
+        <v>0</v>
       </c>
       <c r="G207">
         <v>0</v>
       </c>
       <c r="H207">
-        <v>0.5609603597412309</v>
+        <v>0.5474472275965149</v>
       </c>
       <c r="I207">
-        <v>0.1490265164416418</v>
+        <v>0.1425583099316179</v>
       </c>
     </row>
     <row r="208" spans="1:9">
@@ -6871,10 +6871,10 @@
         <v>0</v>
       </c>
       <c r="H208">
-        <v>0.6038451386425255</v>
+        <v>0.5899789573712763</v>
       </c>
       <c r="I208">
-        <v>0.1118728929202757</v>
+        <v>0.1065714798831008</v>
       </c>
     </row>
     <row r="209" spans="1:9">
@@ -6900,10 +6900,10 @@
         <v>0</v>
       </c>
       <c r="H209">
-        <v>0.5743184850510572</v>
+        <v>0.5645457839187469</v>
       </c>
       <c r="I209">
-        <v>0.1490265164416418</v>
+        <v>0.1426265202151437</v>
       </c>
     </row>
     <row r="210" spans="1:9">
@@ -6929,10 +6929,10 @@
         <v>0</v>
       </c>
       <c r="H210">
-        <v>0.5743184850510572</v>
+        <v>0.5645457839187469</v>
       </c>
       <c r="I210">
-        <v>0.1490265164416418</v>
+        <v>0.1426265202151437</v>
       </c>
     </row>
     <row r="211" spans="1:9">
@@ -6958,10 +6958,10 @@
         <v>0</v>
       </c>
       <c r="H211">
-        <v>0.6193974201557383</v>
+        <v>0.6099090717422234</v>
       </c>
       <c r="I211">
-        <v>0.1118728929202757</v>
+        <v>0.1066275182532352</v>
       </c>
     </row>
     <row r="212" spans="1:9">
@@ -6987,10 +6987,10 @@
         <v>0</v>
       </c>
       <c r="H212">
-        <v>0.5609603597412309</v>
+        <v>0.5474472275965149</v>
       </c>
       <c r="I212">
-        <v>0.1490265164416418</v>
+        <v>0.1426265202151437</v>
       </c>
     </row>
     <row r="213" spans="1:9">
@@ -7016,10 +7016,10 @@
         <v>0</v>
       </c>
       <c r="H213">
-        <v>0.5609603597412309</v>
+        <v>0.5474472275965149</v>
       </c>
       <c r="I213">
-        <v>0.1490265164416418</v>
+        <v>0.1426265202151437</v>
       </c>
     </row>
     <row r="214" spans="1:9">
@@ -7045,10 +7045,10 @@
         <v>0</v>
       </c>
       <c r="H214">
-        <v>0.6038451386425255</v>
+        <v>0.5899789573712763</v>
       </c>
       <c r="I214">
-        <v>0.1118728929202757</v>
+        <v>0.1066275182532352</v>
       </c>
     </row>
     <row r="215" spans="1:9">
@@ -7074,10 +7074,10 @@
         <v>0</v>
       </c>
       <c r="H215">
-        <v>0.5609603597412309</v>
+        <v>0.5474472275965149</v>
       </c>
       <c r="I215">
-        <v>0.1490265164416418</v>
+        <v>0.1426265202151437</v>
       </c>
     </row>
     <row r="216" spans="1:9">
@@ -7103,10 +7103,10 @@
         <v>0</v>
       </c>
       <c r="H216">
-        <v>0.5609603597412309</v>
+        <v>0.5474472275965149</v>
       </c>
       <c r="I216">
-        <v>0.1490265164416418</v>
+        <v>0.1426265202151437</v>
       </c>
     </row>
     <row r="217" spans="1:9">
@@ -7132,10 +7132,10 @@
         <v>0</v>
       </c>
       <c r="H217">
-        <v>0.6038451386425255</v>
+        <v>0.5899789573712763</v>
       </c>
       <c r="I217">
-        <v>0.1118728929202757</v>
+        <v>0.1066275182532352</v>
       </c>
     </row>
     <row r="218" spans="1:9">
@@ -7161,10 +7161,10 @@
         <v>0</v>
       </c>
       <c r="H218">
-        <v>0.5609603597412309</v>
+        <v>0.5474472275965149</v>
       </c>
       <c r="I218">
-        <v>0.1490265164416418</v>
+        <v>0.1426265202151437</v>
       </c>
     </row>
     <row r="219" spans="1:9">
@@ -7190,10 +7190,10 @@
         <v>0</v>
       </c>
       <c r="H219">
-        <v>0.5609603597412309</v>
+        <v>0.5474472275965149</v>
       </c>
       <c r="I219">
-        <v>0.1490265164416418</v>
+        <v>0.1426265202151437</v>
       </c>
     </row>
     <row r="220" spans="1:9">
@@ -7219,10 +7219,10 @@
         <v>0</v>
       </c>
       <c r="H220">
-        <v>0.607661787116463</v>
+        <v>0.592782893328202</v>
       </c>
       <c r="I220">
-        <v>0.1118728929202757</v>
+        <v>0.1066275182532352</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Regenerate all outputs from the merged pipeline
The four integrated branches changed code without regenerating figures, so
the committed outputs were stale against the merged tree. Full Run_All.R +
Compose_Figure_Panels.R run, both clean.

Also drops the logMME composite's orphaned files: mme-panel-into-roe stopped
producing Composite_Fig1 and moved its NRS panel onto the logROE figure, so
those PNG/TIFF/DOCX were left behind on disk. A stray tracked Word lock file
(~$mposite_Fig1_...docx) goes with them.

Known issue, untouched: the overlay figures clip their axis title and legend
at the device edge. That comes from fix-config-caching's longer group names
and larger strip text, and went unnoticed because that branch never
regenerated figures to look at.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/New_Outputs/Figure_StatsBox_Placement_Audit.xlsx
+++ b/New_Outputs/Figure_StatsBox_Placement_Audit.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="666" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="684" uniqueCount="165">
   <si>
     <t>figure</t>
   </si>
@@ -497,6 +497,18 @@
   </si>
   <si>
     <t>Fig_logROE_vs_PC3_overlay</t>
+  </si>
+  <si>
+    <t>Fig_MME_vs_ROE_faceted</t>
+  </si>
+  <si>
+    <t>Fig_MME_vs_ROE_overlay</t>
+  </si>
+  <si>
+    <t>Fig_logMME_vs_logROE_faceted</t>
+  </si>
+  <si>
+    <t>Fig_logMME_vs_logROE_overlay</t>
   </si>
 </sst>
 </file>
@@ -839,7 +851,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I220"/>
+  <dimension ref="A1:I226"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:9" s="1" customFormat="1">
@@ -7222,6 +7234,180 @@
         <v>0.2884950415976383</v>
       </c>
     </row>
+    <row r="221" spans="1:9">
+      <c r="A221" t="s">
+        <v>161</v>
+      </c>
+      <c r="B221" t="s">
+        <v>10</v>
+      </c>
+      <c r="C221" t="s">
+        <v>11</v>
+      </c>
+      <c r="D221">
+        <v>0</v>
+      </c>
+      <c r="E221">
+        <v>0</v>
+      </c>
+      <c r="F221">
+        <v>0.01627192734084503</v>
+      </c>
+      <c r="G221">
+        <v>0</v>
+      </c>
+      <c r="H221">
+        <v>0.5232507257575485</v>
+      </c>
+      <c r="I221">
+        <v>0.3356561405743864</v>
+      </c>
+    </row>
+    <row r="222" spans="1:9">
+      <c r="A222" t="s">
+        <v>161</v>
+      </c>
+      <c r="B222" t="s">
+        <v>12</v>
+      </c>
+      <c r="C222" t="s">
+        <v>11</v>
+      </c>
+      <c r="D222">
+        <v>0</v>
+      </c>
+      <c r="E222">
+        <v>0</v>
+      </c>
+      <c r="F222">
+        <v>0.01627192734084503</v>
+      </c>
+      <c r="G222">
+        <v>0</v>
+      </c>
+      <c r="H222">
+        <v>0.5232507257575485</v>
+      </c>
+      <c r="I222">
+        <v>0.3356561405743864</v>
+      </c>
+    </row>
+    <row r="223" spans="1:9">
+      <c r="A223" t="s">
+        <v>162</v>
+      </c>
+      <c r="B223" t="s">
+        <v>14</v>
+      </c>
+      <c r="C223" t="s">
+        <v>11</v>
+      </c>
+      <c r="D223">
+        <v>0</v>
+      </c>
+      <c r="E223">
+        <v>0</v>
+      </c>
+      <c r="F223">
+        <v>0.012120338378827</v>
+      </c>
+      <c r="G223">
+        <v>0</v>
+      </c>
+      <c r="H223">
+        <v>0.9</v>
+      </c>
+      <c r="I223">
+        <v>0.2773301819958656</v>
+      </c>
+    </row>
+    <row r="224" spans="1:9">
+      <c r="A224" t="s">
+        <v>163</v>
+      </c>
+      <c r="B224" t="s">
+        <v>10</v>
+      </c>
+      <c r="C224" t="s">
+        <v>16</v>
+      </c>
+      <c r="D224">
+        <v>0</v>
+      </c>
+      <c r="E224">
+        <v>0</v>
+      </c>
+      <c r="F224">
+        <v>0</v>
+      </c>
+      <c r="G224">
+        <v>1.812232359039491</v>
+      </c>
+      <c r="H224">
+        <v>0.9</v>
+      </c>
+      <c r="I224">
+        <v>0.3466958044956942</v>
+      </c>
+    </row>
+    <row r="225" spans="1:9">
+      <c r="A225" t="s">
+        <v>163</v>
+      </c>
+      <c r="B225" t="s">
+        <v>12</v>
+      </c>
+      <c r="C225" t="s">
+        <v>11</v>
+      </c>
+      <c r="D225">
+        <v>0</v>
+      </c>
+      <c r="E225">
+        <v>0</v>
+      </c>
+      <c r="F225">
+        <v>0</v>
+      </c>
+      <c r="G225">
+        <v>1.812232359039491</v>
+      </c>
+      <c r="H225">
+        <v>0.9</v>
+      </c>
+      <c r="I225">
+        <v>0.3466958044956942</v>
+      </c>
+    </row>
+    <row r="226" spans="1:9">
+      <c r="A226" t="s">
+        <v>164</v>
+      </c>
+      <c r="B226" t="s">
+        <v>14</v>
+      </c>
+      <c r="C226" t="s">
+        <v>11</v>
+      </c>
+      <c r="D226">
+        <v>0</v>
+      </c>
+      <c r="E226">
+        <v>0</v>
+      </c>
+      <c r="F226">
+        <v>1.356963917722085</v>
+      </c>
+      <c r="G226">
+        <v>0</v>
+      </c>
+      <c r="H226">
+        <v>0.9</v>
+      </c>
+      <c r="I226">
+        <v>0.2884950415976383</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Snapshot before ROE zero-imputation change
Full working-tree snapshot (code + regenerated outputs) taken immediately
before switching log_ROE's zero-handling from complete-case drop to a
2-decades-below-minimum imputation. Kept as the reproducibility baseline
for the old (drop-zeros) behaviour.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/New_Outputs/Figure_StatsBox_Placement_Audit.xlsx
+++ b/New_Outputs/Figure_StatsBox_Placement_Audit.xlsx
@@ -142,25 +142,25 @@
     <t>Fig1_PC3_HT1A_Only</t>
   </si>
   <si>
+    <t>Fig1_PC3_HT1A_Only_overlay</t>
+  </si>
+  <si>
+    <t>Fig1_SOWS_HT1A_Only</t>
+  </si>
+  <si>
+    <t>Fig1_SOWS_HT1A_Only_overlay</t>
+  </si>
+  <si>
+    <t>Fig1_NRS_HT2A_Only</t>
+  </si>
+  <si>
+    <t>Fig1_NRS_HT2A_Only_overlay</t>
+  </si>
+  <si>
+    <t>Fig1_PC1_HT2A_Only</t>
+  </si>
+  <si>
     <t>bottomright</t>
-  </si>
-  <si>
-    <t>Fig1_PC3_HT1A_Only_overlay</t>
-  </si>
-  <si>
-    <t>Fig1_SOWS_HT1A_Only</t>
-  </si>
-  <si>
-    <t>Fig1_SOWS_HT1A_Only_overlay</t>
-  </si>
-  <si>
-    <t>Fig1_NRS_HT2A_Only</t>
-  </si>
-  <si>
-    <t>Fig1_NRS_HT2A_Only_overlay</t>
-  </si>
-  <si>
-    <t>Fig1_PC1_HT2A_Only</t>
   </si>
   <si>
     <t>Fig1_PC1_HT2A_Only_overlay</t>
@@ -903,16 +903,16 @@
         <v>0</v>
       </c>
       <c r="F2">
-        <v>2.30667808136484</v>
+        <v>2.303712824888164</v>
       </c>
       <c r="G2">
         <v>0</v>
       </c>
       <c r="H2">
-        <v>0.7511796927795087</v>
+        <v>0.7652770917997694</v>
       </c>
       <c r="I2">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -932,16 +932,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>2.30667808136484</v>
+        <v>2.303712824888164</v>
       </c>
       <c r="G3">
         <v>0</v>
       </c>
       <c r="H3">
-        <v>0.7511796927795087</v>
+        <v>0.7652770917997694</v>
       </c>
       <c r="I3">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -961,7 +961,7 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>1.806428885364793</v>
+        <v>1.801714163093838</v>
       </c>
       <c r="G4">
         <v>0</v>
@@ -970,7 +970,7 @@
         <v>0.9</v>
       </c>
       <c r="I4">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -996,10 +996,10 @@
         <v>0</v>
       </c>
       <c r="H5">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I5">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -1025,10 +1025,10 @@
         <v>0</v>
       </c>
       <c r="H6">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I6">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -1057,7 +1057,7 @@
         <v>0.9</v>
       </c>
       <c r="I7">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -1077,16 +1077,16 @@
         <v>0</v>
       </c>
       <c r="F8">
-        <v>1.032817216652524</v>
+        <v>1.031489520358167</v>
       </c>
       <c r="G8">
         <v>0</v>
       </c>
       <c r="H8">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I8">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -1106,16 +1106,16 @@
         <v>0</v>
       </c>
       <c r="F9">
-        <v>1.032817216652524</v>
+        <v>1.031489520358167</v>
       </c>
       <c r="G9">
         <v>0</v>
       </c>
       <c r="H9">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I9">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -1135,7 +1135,7 @@
         <v>0</v>
       </c>
       <c r="F10">
-        <v>0.8088301824757718</v>
+        <v>0.8067191612749736</v>
       </c>
       <c r="G10">
         <v>0</v>
@@ -1144,7 +1144,7 @@
         <v>0.9</v>
       </c>
       <c r="I10">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -1167,13 +1167,13 @@
         <v>0</v>
       </c>
       <c r="G11">
-        <v>1.314701839907713</v>
+        <v>1.313011778265744</v>
       </c>
       <c r="H11">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I11">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -1196,13 +1196,13 @@
         <v>0</v>
       </c>
       <c r="G12">
-        <v>1.314701839907713</v>
+        <v>1.313011778265744</v>
       </c>
       <c r="H12">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I12">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -1225,13 +1225,13 @@
         <v>0</v>
       </c>
       <c r="G13">
-        <v>1.029582497201481</v>
+        <v>1.026895319439506</v>
       </c>
       <c r="H13">
         <v>0.9</v>
       </c>
       <c r="I13">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -1257,10 +1257,10 @@
         <v>0</v>
       </c>
       <c r="H14">
-        <v>0.7658084128556363</v>
+        <v>0.7795009861990785</v>
       </c>
       <c r="I14">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="15" spans="1:9">
@@ -1286,10 +1286,10 @@
         <v>0</v>
       </c>
       <c r="H15">
-        <v>0.7658084128556363</v>
+        <v>0.7795009861990785</v>
       </c>
       <c r="I15">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="16" spans="1:9">
@@ -1318,7 +1318,7 @@
         <v>0.9</v>
       </c>
       <c r="I16">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="17" spans="1:9">
@@ -1341,13 +1341,13 @@
         <v>0</v>
       </c>
       <c r="G17">
-        <v>2.306678081364841</v>
+        <v>2.303712824888164</v>
       </c>
       <c r="H17">
-        <v>0.7171704480218883</v>
+        <v>0.7313302934646828</v>
       </c>
       <c r="I17">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="18" spans="1:9">
@@ -1370,13 +1370,13 @@
         <v>0</v>
       </c>
       <c r="G18">
-        <v>2.306678081364841</v>
+        <v>2.303712824888164</v>
       </c>
       <c r="H18">
-        <v>0.7171704480218883</v>
+        <v>0.7313302934646828</v>
       </c>
       <c r="I18">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="19" spans="1:9">
@@ -1396,7 +1396,7 @@
         <v>0</v>
       </c>
       <c r="F19">
-        <v>1.806428885364793</v>
+        <v>1.801714163093838</v>
       </c>
       <c r="G19">
         <v>0</v>
@@ -1405,7 +1405,7 @@
         <v>0.9</v>
       </c>
       <c r="I19">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="20" spans="1:9">
@@ -1431,10 +1431,10 @@
         <v>0</v>
       </c>
       <c r="H20">
-        <v>0.6751324872921075</v>
+        <v>0.6790690123961114</v>
       </c>
       <c r="I20">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="21" spans="1:9">
@@ -1460,10 +1460,10 @@
         <v>0</v>
       </c>
       <c r="H21">
-        <v>0.6751324872921075</v>
+        <v>0.6790690123961114</v>
       </c>
       <c r="I21">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="22" spans="1:9">
@@ -1486,13 +1486,13 @@
         <v>0</v>
       </c>
       <c r="G22">
-        <v>0.9095525618320601</v>
+        <v>0.9071786584060151</v>
       </c>
       <c r="H22">
         <v>0.9</v>
       </c>
       <c r="I22">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="23" spans="1:9">
@@ -1512,16 +1512,16 @@
         <v>0</v>
       </c>
       <c r="F23">
-        <v>1.032817216652524</v>
+        <v>1.031489520358167</v>
       </c>
       <c r="G23">
         <v>0</v>
       </c>
       <c r="H23">
-        <v>0.6751324872921075</v>
+        <v>0.6790690123961114</v>
       </c>
       <c r="I23">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="24" spans="1:9">
@@ -1541,16 +1541,16 @@
         <v>0</v>
       </c>
       <c r="F24">
-        <v>1.032817216652524</v>
+        <v>1.031489520358167</v>
       </c>
       <c r="G24">
         <v>0</v>
       </c>
       <c r="H24">
-        <v>0.6751324872921075</v>
+        <v>0.6790690123961114</v>
       </c>
       <c r="I24">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="25" spans="1:9">
@@ -1570,7 +1570,7 @@
         <v>0</v>
       </c>
       <c r="F25">
-        <v>0.8088301824757718</v>
+        <v>0.8067191612749736</v>
       </c>
       <c r="G25">
         <v>0</v>
@@ -1579,7 +1579,7 @@
         <v>0.9</v>
       </c>
       <c r="I25">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="26" spans="1:9">
@@ -1605,10 +1605,10 @@
         <v>0</v>
       </c>
       <c r="H26">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I26">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="27" spans="1:9">
@@ -1634,10 +1634,10 @@
         <v>0</v>
       </c>
       <c r="H27">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I27">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="28" spans="1:9">
@@ -1660,13 +1660,13 @@
         <v>0</v>
       </c>
       <c r="G28">
-        <v>1.029582497201481</v>
+        <v>1.026895319439506</v>
       </c>
       <c r="H28">
         <v>0.9</v>
       </c>
       <c r="I28">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="29" spans="1:9">
@@ -1686,16 +1686,16 @@
         <v>0</v>
       </c>
       <c r="F29">
-        <v>11.27709284222811</v>
+        <v>11.26259603278658</v>
       </c>
       <c r="G29">
         <v>0</v>
       </c>
       <c r="H29">
-        <v>0.6994687982605935</v>
+        <v>0.7132828385507737</v>
       </c>
       <c r="I29">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="30" spans="1:9">
@@ -1715,16 +1715,16 @@
         <v>0</v>
       </c>
       <c r="F30">
-        <v>11.27709284222811</v>
+        <v>11.26259603278658</v>
       </c>
       <c r="G30">
         <v>0</v>
       </c>
       <c r="H30">
-        <v>0.6994687982605935</v>
+        <v>0.7132828385507737</v>
       </c>
       <c r="I30">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="31" spans="1:9">
@@ -1744,7 +1744,7 @@
         <v>0</v>
       </c>
       <c r="F31">
-        <v>8.831430106227877</v>
+        <v>8.808380352903214</v>
       </c>
       <c r="G31">
         <v>0</v>
@@ -1753,7 +1753,7 @@
         <v>0.9</v>
       </c>
       <c r="I31">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="32" spans="1:9">
@@ -1776,13 +1776,13 @@
         <v>0</v>
       </c>
       <c r="G32">
-        <v>2.306678081364841</v>
+        <v>2.303712824888164</v>
       </c>
       <c r="H32">
-        <v>0.7171704480218883</v>
+        <v>0.7313302934646828</v>
       </c>
       <c r="I32">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="33" spans="1:9">
@@ -1805,13 +1805,13 @@
         <v>0</v>
       </c>
       <c r="G33">
-        <v>2.306678081364841</v>
+        <v>2.303712824888164</v>
       </c>
       <c r="H33">
-        <v>0.7171704480218883</v>
+        <v>0.7313302934646828</v>
       </c>
       <c r="I33">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="34" spans="1:9">
@@ -1831,7 +1831,7 @@
         <v>0</v>
       </c>
       <c r="F34">
-        <v>1.806428885364793</v>
+        <v>1.801714163093838</v>
       </c>
       <c r="G34">
         <v>0</v>
@@ -1840,7 +1840,7 @@
         <v>0.9</v>
       </c>
       <c r="I34">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="35" spans="1:9">
@@ -1866,10 +1866,10 @@
         <v>0</v>
       </c>
       <c r="H35">
-        <v>0.6751324872921075</v>
+        <v>0.6790690123961114</v>
       </c>
       <c r="I35">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="36" spans="1:9">
@@ -1895,10 +1895,10 @@
         <v>0</v>
       </c>
       <c r="H36">
-        <v>0.6751324872921075</v>
+        <v>0.6790690123961114</v>
       </c>
       <c r="I36">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="37" spans="1:9">
@@ -1921,13 +1921,13 @@
         <v>0</v>
       </c>
       <c r="G37">
-        <v>0.9095525618320601</v>
+        <v>0.9071786584060151</v>
       </c>
       <c r="H37">
         <v>0.9</v>
       </c>
       <c r="I37">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="38" spans="1:9">
@@ -1947,16 +1947,16 @@
         <v>0</v>
       </c>
       <c r="F38">
-        <v>1.032817216652524</v>
+        <v>1.031489520358167</v>
       </c>
       <c r="G38">
         <v>0</v>
       </c>
       <c r="H38">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I38">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="39" spans="1:9">
@@ -1976,16 +1976,16 @@
         <v>0</v>
       </c>
       <c r="F39">
-        <v>1.032817216652524</v>
+        <v>1.031489520358167</v>
       </c>
       <c r="G39">
         <v>0</v>
       </c>
       <c r="H39">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I39">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="40" spans="1:9">
@@ -2005,7 +2005,7 @@
         <v>0</v>
       </c>
       <c r="F40">
-        <v>0.8088301824757718</v>
+        <v>0.8067191612749736</v>
       </c>
       <c r="G40">
         <v>0</v>
@@ -2014,7 +2014,7 @@
         <v>0.9</v>
       </c>
       <c r="I40">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="41" spans="1:9">
@@ -2025,7 +2025,7 @@
         <v>10</v>
       </c>
       <c r="C41" t="s">
-        <v>42</v>
+        <v>16</v>
       </c>
       <c r="D41">
         <v>0</v>
@@ -2037,13 +2037,13 @@
         <v>0</v>
       </c>
       <c r="G41">
-        <v>0</v>
+        <v>1.313011778265744</v>
       </c>
       <c r="H41">
-        <v>0.6916236538556428</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I41">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="42" spans="1:9">
@@ -2066,18 +2066,18 @@
         <v>0</v>
       </c>
       <c r="G42">
-        <v>0</v>
+        <v>1.313011778265744</v>
       </c>
       <c r="H42">
-        <v>0.6916236538556428</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I42">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="43" spans="1:9">
       <c r="A43" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B43" t="s">
         <v>14</v>
@@ -2095,18 +2095,18 @@
         <v>0</v>
       </c>
       <c r="G43">
-        <v>1.029582497201481</v>
+        <v>1.026895319439506</v>
       </c>
       <c r="H43">
         <v>0.9</v>
       </c>
       <c r="I43">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="44" spans="1:9">
       <c r="A44" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B44" t="s">
         <v>10</v>
@@ -2121,21 +2121,21 @@
         <v>0</v>
       </c>
       <c r="F44">
-        <v>11.44956844458132</v>
+        <v>11.4348499161227</v>
       </c>
       <c r="G44">
         <v>0</v>
       </c>
       <c r="H44">
-        <v>0.6994687982605935</v>
+        <v>0.7132828385507737</v>
       </c>
       <c r="I44">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="45" spans="1:9">
       <c r="A45" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B45" t="s">
         <v>12</v>
@@ -2150,21 +2150,21 @@
         <v>0</v>
       </c>
       <c r="F45">
-        <v>11.44956844458132</v>
+        <v>11.4348499161227</v>
       </c>
       <c r="G45">
         <v>0</v>
       </c>
       <c r="H45">
-        <v>0.6994687982605935</v>
+        <v>0.7132828385507737</v>
       </c>
       <c r="I45">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="46" spans="1:9">
       <c r="A46" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B46" t="s">
         <v>14</v>
@@ -2179,7 +2179,7 @@
         <v>0</v>
       </c>
       <c r="F46">
-        <v>8.966500930643562</v>
+        <v>8.94309864673815</v>
       </c>
       <c r="G46">
         <v>0</v>
@@ -2188,12 +2188,12 @@
         <v>0.9</v>
       </c>
       <c r="I46">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="47" spans="1:9">
       <c r="A47" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B47" t="s">
         <v>10</v>
@@ -2214,15 +2214,15 @@
         <v>0</v>
       </c>
       <c r="H47">
-        <v>0.7171704480218883</v>
+        <v>0.7313302934646828</v>
       </c>
       <c r="I47">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="48" spans="1:9">
       <c r="A48" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B48" t="s">
         <v>12</v>
@@ -2243,15 +2243,15 @@
         <v>0</v>
       </c>
       <c r="H48">
-        <v>0.7171704480218883</v>
+        <v>0.7313302934646828</v>
       </c>
       <c r="I48">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="49" spans="1:9">
       <c r="A49" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B49" t="s">
         <v>14</v>
@@ -2266,7 +2266,7 @@
         <v>0</v>
       </c>
       <c r="F49">
-        <v>1.806428885364793</v>
+        <v>1.801714163093838</v>
       </c>
       <c r="G49">
         <v>0</v>
@@ -2275,12 +2275,12 @@
         <v>0.9</v>
       </c>
       <c r="I49">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="50" spans="1:9">
       <c r="A50" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B50" t="s">
         <v>10</v>
@@ -2301,21 +2301,21 @@
         <v>0</v>
       </c>
       <c r="H50">
-        <v>0.6751324872921075</v>
+        <v>0.6790690123961114</v>
       </c>
       <c r="I50">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="51" spans="1:9">
       <c r="A51" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B51" t="s">
         <v>12</v>
       </c>
       <c r="C51" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="D51">
         <v>0</v>
@@ -2330,10 +2330,10 @@
         <v>0</v>
       </c>
       <c r="H51">
-        <v>0.6751324872921075</v>
+        <v>0.6790690123961114</v>
       </c>
       <c r="I51">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="52" spans="1:9">
@@ -2356,13 +2356,13 @@
         <v>0</v>
       </c>
       <c r="G52">
-        <v>0.9095525618320601</v>
+        <v>0.9071786584060151</v>
       </c>
       <c r="H52">
         <v>0.9</v>
       </c>
       <c r="I52">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="53" spans="1:9">
@@ -2373,7 +2373,7 @@
         <v>10</v>
       </c>
       <c r="C53" t="s">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="D53">
         <v>0</v>
@@ -2382,16 +2382,16 @@
         <v>0</v>
       </c>
       <c r="F53">
-        <v>0</v>
+        <v>1.031489520358167</v>
       </c>
       <c r="G53">
         <v>0</v>
       </c>
       <c r="H53">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I53">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="54" spans="1:9">
@@ -2402,7 +2402,7 @@
         <v>12</v>
       </c>
       <c r="C54" t="s">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="D54">
         <v>0</v>
@@ -2411,16 +2411,16 @@
         <v>0</v>
       </c>
       <c r="F54">
-        <v>0</v>
+        <v>1.031489520358167</v>
       </c>
       <c r="G54">
         <v>0</v>
       </c>
       <c r="H54">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I54">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="55" spans="1:9">
@@ -2440,7 +2440,7 @@
         <v>0</v>
       </c>
       <c r="F55">
-        <v>0.8088301824757718</v>
+        <v>0.8067191612749736</v>
       </c>
       <c r="G55">
         <v>0</v>
@@ -2449,7 +2449,7 @@
         <v>0.9</v>
       </c>
       <c r="I55">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="56" spans="1:9">
@@ -2472,13 +2472,13 @@
         <v>0</v>
       </c>
       <c r="G56">
-        <v>1.351069916818218</v>
+        <v>1.349333103669624</v>
       </c>
       <c r="H56">
-        <v>0.6751324872921075</v>
+        <v>0.6790690123961114</v>
       </c>
       <c r="I56">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="57" spans="1:9">
@@ -2501,13 +2501,13 @@
         <v>0</v>
       </c>
       <c r="G57">
-        <v>1.351069916818218</v>
+        <v>1.349333103669624</v>
       </c>
       <c r="H57">
-        <v>0.6751324872921075</v>
+        <v>0.6790690123961114</v>
       </c>
       <c r="I57">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="58" spans="1:9">
@@ -2527,7 +2527,7 @@
         <v>0</v>
       </c>
       <c r="F58">
-        <v>1.058063430525923</v>
+        <v>1.055301918428547</v>
       </c>
       <c r="G58">
         <v>0</v>
@@ -2536,7 +2536,7 @@
         <v>0.9</v>
       </c>
       <c r="I58">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="59" spans="1:9">
@@ -2562,10 +2562,10 @@
         <v>0</v>
       </c>
       <c r="H59">
-        <v>0.7064311782928777</v>
+        <v>0.7258252566857329</v>
       </c>
       <c r="I59">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="60" spans="1:9">
@@ -2591,10 +2591,10 @@
         <v>0</v>
       </c>
       <c r="H60">
-        <v>0.7064311782928777</v>
+        <v>0.7258252566857329</v>
       </c>
       <c r="I60">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="61" spans="1:9">
@@ -2623,7 +2623,7 @@
         <v>0.9</v>
       </c>
       <c r="I61">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="62" spans="1:9">
@@ -2646,13 +2646,13 @@
         <v>0</v>
       </c>
       <c r="G62">
-        <v>2.36239619379422</v>
+        <v>2.359359311157359</v>
       </c>
       <c r="H62">
-        <v>0.7171704480218883</v>
+        <v>0.7313302934646828</v>
       </c>
       <c r="I62">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="63" spans="1:9">
@@ -2675,13 +2675,13 @@
         <v>0</v>
       </c>
       <c r="G63">
-        <v>2.36239619379422</v>
+        <v>2.359359311157359</v>
       </c>
       <c r="H63">
-        <v>0.7171704480218883</v>
+        <v>0.7313302934646828</v>
       </c>
       <c r="I63">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="64" spans="1:9">
@@ -2701,7 +2701,7 @@
         <v>0</v>
       </c>
       <c r="F64">
-        <v>1.85006341267208</v>
+        <v>1.845234805664591</v>
       </c>
       <c r="G64">
         <v>0</v>
@@ -2710,7 +2710,7 @@
         <v>0.9</v>
       </c>
       <c r="I64">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="65" spans="1:9">
@@ -2730,16 +2730,16 @@
         <v>0</v>
       </c>
       <c r="F65">
-        <v>1.161432357080345</v>
+        <v>1.159939324807278</v>
       </c>
       <c r="G65">
         <v>0</v>
       </c>
       <c r="H65">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I65">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="66" spans="1:9">
@@ -2759,16 +2759,16 @@
         <v>0</v>
       </c>
       <c r="F66">
-        <v>1.161432357080345</v>
+        <v>1.159939324807278</v>
       </c>
       <c r="G66">
         <v>0</v>
       </c>
       <c r="H66">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I66">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="67" spans="1:9">
@@ -2791,13 +2791,13 @@
         <v>0</v>
       </c>
       <c r="G67">
-        <v>0.9095525618320601</v>
+        <v>0.9071786584060151</v>
       </c>
       <c r="H67">
         <v>0.9</v>
       </c>
       <c r="I67">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="68" spans="1:9">
@@ -2817,16 +2817,16 @@
         <v>0</v>
       </c>
       <c r="F68">
-        <v>1.032817216652524</v>
+        <v>1.031489520358167</v>
       </c>
       <c r="G68">
         <v>0</v>
       </c>
       <c r="H68">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I68">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="69" spans="1:9">
@@ -2846,16 +2846,16 @@
         <v>0</v>
       </c>
       <c r="F69">
-        <v>1.032817216652524</v>
+        <v>1.031489520358167</v>
       </c>
       <c r="G69">
         <v>0</v>
       </c>
       <c r="H69">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I69">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="70" spans="1:9">
@@ -2875,7 +2875,7 @@
         <v>0</v>
       </c>
       <c r="F70">
-        <v>0.8088301824757718</v>
+        <v>0.8067191612749736</v>
       </c>
       <c r="G70">
         <v>0</v>
@@ -2884,7 +2884,7 @@
         <v>0.9</v>
       </c>
       <c r="I70">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="71" spans="1:9">
@@ -2907,13 +2907,13 @@
         <v>0</v>
       </c>
       <c r="G71">
-        <v>1.314701839907713</v>
+        <v>1.313011778265744</v>
       </c>
       <c r="H71">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I71">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="72" spans="1:9">
@@ -2936,13 +2936,13 @@
         <v>0</v>
       </c>
       <c r="G72">
-        <v>1.314701839907713</v>
+        <v>1.313011778265744</v>
       </c>
       <c r="H72">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I72">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="73" spans="1:9">
@@ -2965,13 +2965,13 @@
         <v>0</v>
       </c>
       <c r="G73">
-        <v>1.029582497201481</v>
+        <v>1.026895319439506</v>
       </c>
       <c r="H73">
         <v>0.9</v>
       </c>
       <c r="I73">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="74" spans="1:9">
@@ -2997,10 +2997,10 @@
         <v>0</v>
       </c>
       <c r="H74">
-        <v>0.7127609991721345</v>
+        <v>0.7116154751207804</v>
       </c>
       <c r="I74">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="75" spans="1:9">
@@ -3026,10 +3026,10 @@
         <v>0</v>
       </c>
       <c r="H75">
-        <v>0.7127609991721345</v>
+        <v>0.7116154751207804</v>
       </c>
       <c r="I75">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="76" spans="1:9">
@@ -3058,7 +3058,7 @@
         <v>0.9</v>
       </c>
       <c r="I76">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="77" spans="1:9">
@@ -3078,16 +3078,16 @@
         <v>0</v>
       </c>
       <c r="F77">
-        <v>2.370764193828881</v>
+        <v>2.367716554048879</v>
       </c>
       <c r="G77">
         <v>0</v>
       </c>
       <c r="H77">
-        <v>0.6967897935697006</v>
+        <v>0.6956739441343036</v>
       </c>
       <c r="I77">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="78" spans="1:9">
@@ -3107,16 +3107,16 @@
         <v>0</v>
       </c>
       <c r="F78">
-        <v>2.370764193828881</v>
+        <v>2.367716554048879</v>
       </c>
       <c r="G78">
         <v>0</v>
       </c>
       <c r="H78">
-        <v>0.6967897935697006</v>
+        <v>0.6956739441343036</v>
       </c>
       <c r="I78">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="79" spans="1:9">
@@ -3136,7 +3136,7 @@
         <v>0</v>
       </c>
       <c r="F79">
-        <v>1.856616644827648</v>
+        <v>1.851770934091448</v>
       </c>
       <c r="G79">
         <v>0</v>
@@ -3145,7 +3145,7 @@
         <v>0.9</v>
       </c>
       <c r="I79">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="80" spans="1:9">
@@ -3171,10 +3171,10 @@
         <v>0</v>
       </c>
       <c r="H80">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I80">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="81" spans="1:9">
@@ -3200,10 +3200,10 @@
         <v>0</v>
       </c>
       <c r="H81">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I81">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="82" spans="1:9">
@@ -3232,7 +3232,7 @@
         <v>0.9</v>
       </c>
       <c r="I82">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="83" spans="1:9">
@@ -3252,16 +3252,16 @@
         <v>0</v>
       </c>
       <c r="F83">
-        <v>1.032817216652524</v>
+        <v>1.031489520358167</v>
       </c>
       <c r="G83">
         <v>0</v>
       </c>
       <c r="H83">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I83">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="84" spans="1:9">
@@ -3281,16 +3281,16 @@
         <v>0</v>
       </c>
       <c r="F84">
-        <v>1.032817216652524</v>
+        <v>1.031489520358167</v>
       </c>
       <c r="G84">
         <v>0</v>
       </c>
       <c r="H84">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I84">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="85" spans="1:9">
@@ -3310,7 +3310,7 @@
         <v>0</v>
       </c>
       <c r="F85">
-        <v>0.8088301824757718</v>
+        <v>0.8067191612749736</v>
       </c>
       <c r="G85">
         <v>0</v>
@@ -3319,7 +3319,7 @@
         <v>0.9</v>
       </c>
       <c r="I85">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="86" spans="1:9">
@@ -3330,7 +3330,7 @@
         <v>10</v>
       </c>
       <c r="C86" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="D86">
         <v>0</v>
@@ -3345,10 +3345,10 @@
         <v>0</v>
       </c>
       <c r="H86">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I86">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="87" spans="1:9">
@@ -3374,10 +3374,10 @@
         <v>0</v>
       </c>
       <c r="H87">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I87">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="88" spans="1:9">
@@ -3400,13 +3400,13 @@
         <v>0</v>
       </c>
       <c r="G88">
-        <v>1.029582497201481</v>
+        <v>1.026895319439506</v>
       </c>
       <c r="H88">
         <v>0.9</v>
       </c>
       <c r="I88">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="89" spans="1:9">
@@ -3426,16 +3426,16 @@
         <v>0</v>
       </c>
       <c r="F89">
-        <v>11.93791210217439</v>
+        <v>11.92256580332803</v>
       </c>
       <c r="G89">
         <v>0</v>
       </c>
       <c r="H89">
-        <v>0.6994687982605935</v>
+        <v>0.7132828385507737</v>
       </c>
       <c r="I89">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="90" spans="1:9">
@@ -3455,16 +3455,16 @@
         <v>0</v>
       </c>
       <c r="F90">
-        <v>11.93791210217439</v>
+        <v>11.92256580332803</v>
       </c>
       <c r="G90">
         <v>0</v>
       </c>
       <c r="H90">
-        <v>0.6994687982605935</v>
+        <v>0.7132828385507737</v>
       </c>
       <c r="I90">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="91" spans="1:9">
@@ -3484,7 +3484,7 @@
         <v>0</v>
       </c>
       <c r="F91">
-        <v>9.348937516046426</v>
+        <v>9.324537084745884</v>
       </c>
       <c r="G91">
         <v>0</v>
@@ -3493,7 +3493,7 @@
         <v>0.9</v>
       </c>
       <c r="I91">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="92" spans="1:9">
@@ -3516,13 +3516,13 @@
         <v>0</v>
       </c>
       <c r="G92">
-        <v>2.306678081364841</v>
+        <v>2.303712824888164</v>
       </c>
       <c r="H92">
-        <v>0.7171704480218883</v>
+        <v>0.7313302934646828</v>
       </c>
       <c r="I92">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="93" spans="1:9">
@@ -3545,13 +3545,13 @@
         <v>0</v>
       </c>
       <c r="G93">
-        <v>2.306678081364841</v>
+        <v>2.303712824888164</v>
       </c>
       <c r="H93">
-        <v>0.7171704480218883</v>
+        <v>0.7313302934646828</v>
       </c>
       <c r="I93">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="94" spans="1:9">
@@ -3571,7 +3571,7 @@
         <v>0</v>
       </c>
       <c r="F94">
-        <v>1.806428885364793</v>
+        <v>1.801714163093838</v>
       </c>
       <c r="G94">
         <v>0</v>
@@ -3580,7 +3580,7 @@
         <v>0.9</v>
       </c>
       <c r="I94">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="95" spans="1:9">
@@ -3606,10 +3606,10 @@
         <v>0</v>
       </c>
       <c r="H95">
-        <v>0.6916236538556428</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I95">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="96" spans="1:9">
@@ -3635,10 +3635,10 @@
         <v>0</v>
       </c>
       <c r="H96">
-        <v>0.6916236538556428</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I96">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="97" spans="1:9">
@@ -3658,7 +3658,7 @@
         <v>0</v>
       </c>
       <c r="F97">
-        <v>0.9313413156286918</v>
+        <v>0.9289105442442049</v>
       </c>
       <c r="G97">
         <v>0</v>
@@ -3667,7 +3667,7 @@
         <v>0.9</v>
       </c>
       <c r="I97">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="98" spans="1:9">
@@ -3687,16 +3687,16 @@
         <v>0</v>
       </c>
       <c r="F98">
-        <v>1.032817216652524</v>
+        <v>1.031489520358167</v>
       </c>
       <c r="G98">
         <v>0</v>
       </c>
       <c r="H98">
-        <v>0.6751324872921075</v>
+        <v>0.6790690123961114</v>
       </c>
       <c r="I98">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="99" spans="1:9">
@@ -3716,16 +3716,16 @@
         <v>0</v>
       </c>
       <c r="F99">
-        <v>1.032817216652524</v>
+        <v>1.031489520358167</v>
       </c>
       <c r="G99">
         <v>0</v>
       </c>
       <c r="H99">
-        <v>0.6751324872921075</v>
+        <v>0.6790690123961114</v>
       </c>
       <c r="I99">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="100" spans="1:9">
@@ -3745,7 +3745,7 @@
         <v>0</v>
       </c>
       <c r="F100">
-        <v>0.8088301824757718</v>
+        <v>0.8067191612749736</v>
       </c>
       <c r="G100">
         <v>0</v>
@@ -3754,7 +3754,7 @@
         <v>0.9</v>
       </c>
       <c r="I100">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="101" spans="1:9">
@@ -3777,13 +3777,13 @@
         <v>0</v>
       </c>
       <c r="G101">
-        <v>1.314701839907713</v>
+        <v>1.313011778265744</v>
       </c>
       <c r="H101">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I101">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="102" spans="1:9">
@@ -3806,13 +3806,13 @@
         <v>0</v>
       </c>
       <c r="G102">
-        <v>1.314701839907713</v>
+        <v>1.313011778265744</v>
       </c>
       <c r="H102">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I102">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="103" spans="1:9">
@@ -3835,13 +3835,13 @@
         <v>0</v>
       </c>
       <c r="G103">
-        <v>1.029582497201481</v>
+        <v>1.026895319439506</v>
       </c>
       <c r="H103">
         <v>0.9</v>
       </c>
       <c r="I103">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="104" spans="1:9">
@@ -3861,16 +3861,16 @@
         <v>0</v>
       </c>
       <c r="F104">
-        <v>11.27709284222811</v>
+        <v>11.26259603278658</v>
       </c>
       <c r="G104">
         <v>0</v>
       </c>
       <c r="H104">
-        <v>0.6994687982605935</v>
+        <v>0.7132828385507737</v>
       </c>
       <c r="I104">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="105" spans="1:9">
@@ -3890,16 +3890,16 @@
         <v>0</v>
       </c>
       <c r="F105">
-        <v>11.27709284222811</v>
+        <v>11.26259603278658</v>
       </c>
       <c r="G105">
         <v>0</v>
       </c>
       <c r="H105">
-        <v>0.6994687982605935</v>
+        <v>0.7132828385507737</v>
       </c>
       <c r="I105">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="106" spans="1:9">
@@ -3919,7 +3919,7 @@
         <v>0</v>
       </c>
       <c r="F106">
-        <v>8.831430106227877</v>
+        <v>8.808380352903214</v>
       </c>
       <c r="G106">
         <v>0</v>
@@ -3928,7 +3928,7 @@
         <v>0.9</v>
       </c>
       <c r="I106">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="107" spans="1:9">
@@ -3948,16 +3948,16 @@
         <v>0</v>
       </c>
       <c r="F107">
-        <v>2.30667808136484</v>
+        <v>2.303712824888164</v>
       </c>
       <c r="G107">
         <v>0</v>
       </c>
       <c r="H107">
-        <v>0.7171704480218883</v>
+        <v>0.7313302934646828</v>
       </c>
       <c r="I107">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="108" spans="1:9">
@@ -3977,16 +3977,16 @@
         <v>0</v>
       </c>
       <c r="F108">
-        <v>2.30667808136484</v>
+        <v>2.303712824888164</v>
       </c>
       <c r="G108">
         <v>0</v>
       </c>
       <c r="H108">
-        <v>0.7171704480218883</v>
+        <v>0.7313302934646828</v>
       </c>
       <c r="I108">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="109" spans="1:9">
@@ -4006,7 +4006,7 @@
         <v>0</v>
       </c>
       <c r="F109">
-        <v>1.806428885364793</v>
+        <v>1.801714163093838</v>
       </c>
       <c r="G109">
         <v>0</v>
@@ -4015,7 +4015,7 @@
         <v>0.9</v>
       </c>
       <c r="I109">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="110" spans="1:9">
@@ -4041,10 +4041,10 @@
         <v>0</v>
       </c>
       <c r="H110">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I110">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="111" spans="1:9">
@@ -4070,10 +4070,10 @@
         <v>0</v>
       </c>
       <c r="H111">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I111">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="112" spans="1:9">
@@ -4096,13 +4096,13 @@
         <v>0</v>
       </c>
       <c r="G112">
-        <v>0.914487004639442</v>
+        <v>0.9121002224736987</v>
       </c>
       <c r="H112">
         <v>0.9</v>
       </c>
       <c r="I112">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="113" spans="1:9">
@@ -4122,16 +4122,16 @@
         <v>0</v>
       </c>
       <c r="F113">
-        <v>1.032817216652524</v>
+        <v>1.031489520358167</v>
       </c>
       <c r="G113">
         <v>0</v>
       </c>
       <c r="H113">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I113">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="114" spans="1:9">
@@ -4151,16 +4151,16 @@
         <v>0</v>
       </c>
       <c r="F114">
-        <v>1.032817216652524</v>
+        <v>1.031489520358167</v>
       </c>
       <c r="G114">
         <v>0</v>
       </c>
       <c r="H114">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I114">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="115" spans="1:9">
@@ -4180,7 +4180,7 @@
         <v>0</v>
       </c>
       <c r="F115">
-        <v>0.8088301824757718</v>
+        <v>0.8067191612749736</v>
       </c>
       <c r="G115">
         <v>0</v>
@@ -4189,7 +4189,7 @@
         <v>0.9</v>
       </c>
       <c r="I115">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="116" spans="1:9">
@@ -4212,13 +4212,13 @@
         <v>0</v>
       </c>
       <c r="G116">
-        <v>1.314701839907713</v>
+        <v>1.313011778265744</v>
       </c>
       <c r="H116">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I116">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="117" spans="1:9">
@@ -4241,13 +4241,13 @@
         <v>0</v>
       </c>
       <c r="G117">
-        <v>1.314701839907713</v>
+        <v>1.313011778265744</v>
       </c>
       <c r="H117">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I117">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="118" spans="1:9">
@@ -4270,13 +4270,13 @@
         <v>0</v>
       </c>
       <c r="G118">
-        <v>1.029582497201481</v>
+        <v>1.026895319439506</v>
       </c>
       <c r="H118">
         <v>0.9</v>
       </c>
       <c r="I118">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="119" spans="1:9">
@@ -4302,10 +4302,10 @@
         <v>0</v>
       </c>
       <c r="H119">
-        <v>0.6795911918746134</v>
+        <v>0.6785064012966276</v>
       </c>
       <c r="I119">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="120" spans="1:9">
@@ -4331,10 +4331,10 @@
         <v>0</v>
       </c>
       <c r="H120">
-        <v>0.6795911918746134</v>
+        <v>0.6785064012966276</v>
       </c>
       <c r="I120">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="121" spans="1:9">
@@ -4354,7 +4354,7 @@
         <v>0</v>
       </c>
       <c r="F121">
-        <v>9.934498153426667</v>
+        <v>9.908569427378168</v>
       </c>
       <c r="G121">
         <v>0</v>
@@ -4363,7 +4363,7 @@
         <v>0.9</v>
       </c>
       <c r="I121">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="122" spans="1:9">
@@ -4389,10 +4389,10 @@
         <v>0</v>
       </c>
       <c r="H122">
-        <v>0.7171704480218883</v>
+        <v>0.7313302934646828</v>
       </c>
       <c r="I122">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="123" spans="1:9">
@@ -4418,10 +4418,10 @@
         <v>0</v>
       </c>
       <c r="H123">
-        <v>0.7171704480218883</v>
+        <v>0.7313302934646828</v>
       </c>
       <c r="I123">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="124" spans="1:9">
@@ -4441,7 +4441,7 @@
         <v>0</v>
       </c>
       <c r="F124">
-        <v>1.806428885364793</v>
+        <v>1.801714163093838</v>
       </c>
       <c r="G124">
         <v>0</v>
@@ -4450,7 +4450,7 @@
         <v>0.9</v>
       </c>
       <c r="I124">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="125" spans="1:9">
@@ -4470,16 +4470,16 @@
         <v>0</v>
       </c>
       <c r="F125">
-        <v>1.161432357080345</v>
+        <v>1.159939324807278</v>
       </c>
       <c r="G125">
         <v>0</v>
       </c>
       <c r="H125">
-        <v>0.6751324872921075</v>
+        <v>0.6790690123961114</v>
       </c>
       <c r="I125">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="126" spans="1:9">
@@ -4499,16 +4499,16 @@
         <v>0</v>
       </c>
       <c r="F126">
-        <v>1.161432357080345</v>
+        <v>1.159939324807278</v>
       </c>
       <c r="G126">
         <v>0</v>
       </c>
       <c r="H126">
-        <v>0.6751324872921075</v>
+        <v>0.6790690123961114</v>
       </c>
       <c r="I126">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="127" spans="1:9">
@@ -4531,13 +4531,13 @@
         <v>0</v>
       </c>
       <c r="G127">
-        <v>0.9095525618320601</v>
+        <v>0.9071786584060151</v>
       </c>
       <c r="H127">
         <v>0.9</v>
       </c>
       <c r="I127">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="128" spans="1:9">
@@ -4557,16 +4557,16 @@
         <v>0</v>
       </c>
       <c r="F128">
-        <v>1.032817216652524</v>
+        <v>1.031489520358167</v>
       </c>
       <c r="G128">
         <v>0</v>
       </c>
       <c r="H128">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I128">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="129" spans="1:9">
@@ -4586,16 +4586,16 @@
         <v>0</v>
       </c>
       <c r="F129">
-        <v>1.032817216652524</v>
+        <v>1.031489520358167</v>
       </c>
       <c r="G129">
         <v>0</v>
       </c>
       <c r="H129">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I129">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="130" spans="1:9">
@@ -4615,7 +4615,7 @@
         <v>0</v>
       </c>
       <c r="F130">
-        <v>0.8088301824757718</v>
+        <v>0.8067191612749736</v>
       </c>
       <c r="G130">
         <v>0</v>
@@ -4624,7 +4624,7 @@
         <v>0.9</v>
       </c>
       <c r="I130">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="131" spans="1:9">
@@ -4635,7 +4635,7 @@
         <v>10</v>
       </c>
       <c r="C131" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="D131">
         <v>0</v>
@@ -4650,10 +4650,10 @@
         <v>0</v>
       </c>
       <c r="H131">
-        <v>0.6751324872921075</v>
+        <v>0.6790690123961114</v>
       </c>
       <c r="I131">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="132" spans="1:9">
@@ -4664,7 +4664,7 @@
         <v>12</v>
       </c>
       <c r="C132" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="D132">
         <v>0</v>
@@ -4679,10 +4679,10 @@
         <v>0</v>
       </c>
       <c r="H132">
-        <v>0.6751324872921075</v>
+        <v>0.6790690123961114</v>
       </c>
       <c r="I132">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="133" spans="1:9">
@@ -4705,13 +4705,13 @@
         <v>0</v>
       </c>
       <c r="G133">
-        <v>1.029582497201481</v>
+        <v>1.026895319439506</v>
       </c>
       <c r="H133">
         <v>0.9</v>
       </c>
       <c r="I133">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="134" spans="1:9">
@@ -4737,10 +4737,10 @@
         <v>0</v>
       </c>
       <c r="H134">
-        <v>0.7064311782928777</v>
+        <v>0.7258252566857329</v>
       </c>
       <c r="I134">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="135" spans="1:9">
@@ -4766,10 +4766,10 @@
         <v>0</v>
       </c>
       <c r="H135">
-        <v>0.7064311782928777</v>
+        <v>0.7258252566857329</v>
       </c>
       <c r="I135">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="136" spans="1:9">
@@ -4798,7 +4798,7 @@
         <v>0.9</v>
       </c>
       <c r="I136">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="137" spans="1:9">
@@ -4824,10 +4824,10 @@
         <v>0</v>
       </c>
       <c r="H137">
-        <v>0.6967897935697006</v>
+        <v>0.6956739441343036</v>
       </c>
       <c r="I137">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="138" spans="1:9">
@@ -4853,10 +4853,10 @@
         <v>0</v>
       </c>
       <c r="H138">
-        <v>0.6967897935697006</v>
+        <v>0.6956739441343036</v>
       </c>
       <c r="I138">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="139" spans="1:9">
@@ -4876,7 +4876,7 @@
         <v>0</v>
       </c>
       <c r="F139">
-        <v>1.806428885364793</v>
+        <v>1.801714163093838</v>
       </c>
       <c r="G139">
         <v>0</v>
@@ -4885,7 +4885,7 @@
         <v>0.9</v>
       </c>
       <c r="I139">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="140" spans="1:9">
@@ -4911,10 +4911,10 @@
         <v>0</v>
       </c>
       <c r="H140">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I140">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="141" spans="1:9">
@@ -4940,10 +4940,10 @@
         <v>0</v>
       </c>
       <c r="H141">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I141">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="142" spans="1:9">
@@ -4972,7 +4972,7 @@
         <v>0.9</v>
       </c>
       <c r="I142">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="143" spans="1:9">
@@ -4992,16 +4992,16 @@
         <v>0</v>
       </c>
       <c r="F143">
-        <v>1.032817216652524</v>
+        <v>1.031489520358167</v>
       </c>
       <c r="G143">
         <v>0</v>
       </c>
       <c r="H143">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I143">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="144" spans="1:9">
@@ -5021,16 +5021,16 @@
         <v>0</v>
       </c>
       <c r="F144">
-        <v>1.032817216652524</v>
+        <v>1.031489520358167</v>
       </c>
       <c r="G144">
         <v>0</v>
       </c>
       <c r="H144">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I144">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="145" spans="1:9">
@@ -5050,7 +5050,7 @@
         <v>0</v>
       </c>
       <c r="F145">
-        <v>0.8088301824757718</v>
+        <v>0.8067191612749736</v>
       </c>
       <c r="G145">
         <v>0</v>
@@ -5059,7 +5059,7 @@
         <v>0.9</v>
       </c>
       <c r="I145">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="146" spans="1:9">
@@ -5079,16 +5079,16 @@
         <v>0</v>
       </c>
       <c r="F146">
-        <v>1.314701839907713</v>
+        <v>1.313011778265744</v>
       </c>
       <c r="G146">
         <v>0</v>
       </c>
       <c r="H146">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I146">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="147" spans="1:9">
@@ -5108,16 +5108,16 @@
         <v>0</v>
       </c>
       <c r="F147">
-        <v>1.314701839907713</v>
+        <v>1.313011778265744</v>
       </c>
       <c r="G147">
         <v>0</v>
       </c>
       <c r="H147">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I147">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="148" spans="1:9">
@@ -5140,13 +5140,13 @@
         <v>0</v>
       </c>
       <c r="G148">
-        <v>1.029582497201481</v>
+        <v>1.026895319439506</v>
       </c>
       <c r="H148">
         <v>0.9</v>
       </c>
       <c r="I148">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="149" spans="1:9">
@@ -5172,10 +5172,10 @@
         <v>0</v>
       </c>
       <c r="H149">
-        <v>0.7127609991721345</v>
+        <v>0.7132828385507737</v>
       </c>
       <c r="I149">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="150" spans="1:9">
@@ -5201,10 +5201,10 @@
         <v>0</v>
       </c>
       <c r="H150">
-        <v>0.7127609991721345</v>
+        <v>0.7132828385507737</v>
       </c>
       <c r="I150">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="151" spans="1:9">
@@ -5233,7 +5233,7 @@
         <v>0.9</v>
       </c>
       <c r="I151">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="152" spans="1:9">
@@ -5253,16 +5253,16 @@
         <v>0</v>
       </c>
       <c r="F152">
-        <v>2.30667808136484</v>
+        <v>2.303712824888164</v>
       </c>
       <c r="G152">
         <v>0</v>
       </c>
       <c r="H152">
-        <v>0.7171704480218883</v>
+        <v>0.7313302934646828</v>
       </c>
       <c r="I152">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="153" spans="1:9">
@@ -5282,16 +5282,16 @@
         <v>0</v>
       </c>
       <c r="F153">
-        <v>2.30667808136484</v>
+        <v>2.303712824888164</v>
       </c>
       <c r="G153">
         <v>0</v>
       </c>
       <c r="H153">
-        <v>0.7171704480218883</v>
+        <v>0.7313302934646828</v>
       </c>
       <c r="I153">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="154" spans="1:9">
@@ -5311,7 +5311,7 @@
         <v>0</v>
       </c>
       <c r="F154">
-        <v>1.806428885364793</v>
+        <v>1.801714163093838</v>
       </c>
       <c r="G154">
         <v>0</v>
@@ -5320,7 +5320,7 @@
         <v>0.9</v>
       </c>
       <c r="I154">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="155" spans="1:9">
@@ -5346,10 +5346,10 @@
         <v>0</v>
       </c>
       <c r="H155">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I155">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="156" spans="1:9">
@@ -5375,10 +5375,10 @@
         <v>0</v>
       </c>
       <c r="H156">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I156">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="157" spans="1:9">
@@ -5401,13 +5401,13 @@
         <v>0</v>
       </c>
       <c r="G157">
-        <v>0.9095525618320601</v>
+        <v>0.9071786584060151</v>
       </c>
       <c r="H157">
         <v>0.9</v>
       </c>
       <c r="I157">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="158" spans="1:9">
@@ -5427,16 +5427,16 @@
         <v>0</v>
       </c>
       <c r="F158">
-        <v>1.032817216652524</v>
+        <v>1.031489520358167</v>
       </c>
       <c r="G158">
         <v>0</v>
       </c>
       <c r="H158">
-        <v>0.6751324872921075</v>
+        <v>0.6790690123961114</v>
       </c>
       <c r="I158">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="159" spans="1:9">
@@ -5456,16 +5456,16 @@
         <v>0</v>
       </c>
       <c r="F159">
-        <v>1.032817216652524</v>
+        <v>1.031489520358167</v>
       </c>
       <c r="G159">
         <v>0</v>
       </c>
       <c r="H159">
-        <v>0.6751324872921075</v>
+        <v>0.6790690123961114</v>
       </c>
       <c r="I159">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="160" spans="1:9">
@@ -5485,7 +5485,7 @@
         <v>0</v>
       </c>
       <c r="F160">
-        <v>0.8088301824757718</v>
+        <v>0.8067191612749736</v>
       </c>
       <c r="G160">
         <v>0</v>
@@ -5494,7 +5494,7 @@
         <v>0.9</v>
       </c>
       <c r="I160">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="161" spans="1:9">
@@ -5520,10 +5520,10 @@
         <v>0</v>
       </c>
       <c r="H161">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I161">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="162" spans="1:9">
@@ -5549,10 +5549,10 @@
         <v>0</v>
       </c>
       <c r="H162">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I162">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="163" spans="1:9">
@@ -5575,13 +5575,13 @@
         <v>0</v>
       </c>
       <c r="G163">
-        <v>1.029582497201481</v>
+        <v>1.026895319439506</v>
       </c>
       <c r="H163">
         <v>0.9</v>
       </c>
       <c r="I163">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="164" spans="1:9">
@@ -5601,16 +5601,16 @@
         <v>0</v>
       </c>
       <c r="F164">
-        <v>11.27709284222811</v>
+        <v>11.26259603278658</v>
       </c>
       <c r="G164">
         <v>0</v>
       </c>
       <c r="H164">
-        <v>0.6994687982605935</v>
+        <v>0.7132828385507737</v>
       </c>
       <c r="I164">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="165" spans="1:9">
@@ -5630,16 +5630,16 @@
         <v>0</v>
       </c>
       <c r="F165">
-        <v>11.27709284222811</v>
+        <v>11.26259603278658</v>
       </c>
       <c r="G165">
         <v>0</v>
       </c>
       <c r="H165">
-        <v>0.6994687982605935</v>
+        <v>0.7132828385507737</v>
       </c>
       <c r="I165">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="166" spans="1:9">
@@ -5659,7 +5659,7 @@
         <v>0</v>
       </c>
       <c r="F166">
-        <v>8.831430106227877</v>
+        <v>8.808380352903214</v>
       </c>
       <c r="G166">
         <v>0</v>
@@ -5668,7 +5668,7 @@
         <v>0.9</v>
       </c>
       <c r="I166">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="167" spans="1:9">
@@ -5688,16 +5688,16 @@
         <v>0</v>
       </c>
       <c r="F167">
-        <v>2.30667808136484</v>
+        <v>2.303712824888164</v>
       </c>
       <c r="G167">
         <v>0</v>
       </c>
       <c r="H167">
-        <v>0.7171704480218883</v>
+        <v>0.7313302934646828</v>
       </c>
       <c r="I167">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="168" spans="1:9">
@@ -5717,16 +5717,16 @@
         <v>0</v>
       </c>
       <c r="F168">
-        <v>2.30667808136484</v>
+        <v>2.303712824888164</v>
       </c>
       <c r="G168">
         <v>0</v>
       </c>
       <c r="H168">
-        <v>0.7171704480218883</v>
+        <v>0.7313302934646828</v>
       </c>
       <c r="I168">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="169" spans="1:9">
@@ -5746,7 +5746,7 @@
         <v>0</v>
       </c>
       <c r="F169">
-        <v>1.806428885364793</v>
+        <v>1.801714163093838</v>
       </c>
       <c r="G169">
         <v>0</v>
@@ -5755,7 +5755,7 @@
         <v>0.9</v>
       </c>
       <c r="I169">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="170" spans="1:9">
@@ -5781,10 +5781,10 @@
         <v>0</v>
       </c>
       <c r="H170">
-        <v>0.6751324872921075</v>
+        <v>0.6790690123961114</v>
       </c>
       <c r="I170">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="171" spans="1:9">
@@ -5810,10 +5810,10 @@
         <v>0</v>
       </c>
       <c r="H171">
-        <v>0.6751324872921075</v>
+        <v>0.6790690123961114</v>
       </c>
       <c r="I171">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="172" spans="1:9">
@@ -5836,13 +5836,13 @@
         <v>0</v>
       </c>
       <c r="G172">
-        <v>0.9095525618320601</v>
+        <v>0.9071786584060151</v>
       </c>
       <c r="H172">
         <v>0.9</v>
       </c>
       <c r="I172">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="173" spans="1:9">
@@ -5862,16 +5862,16 @@
         <v>0</v>
       </c>
       <c r="F173">
-        <v>1.032817216652524</v>
+        <v>1.031489520358167</v>
       </c>
       <c r="G173">
         <v>0</v>
       </c>
       <c r="H173">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I173">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="174" spans="1:9">
@@ -5891,16 +5891,16 @@
         <v>0</v>
       </c>
       <c r="F174">
-        <v>1.032817216652524</v>
+        <v>1.031489520358167</v>
       </c>
       <c r="G174">
         <v>0</v>
       </c>
       <c r="H174">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I174">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="175" spans="1:9">
@@ -5920,7 +5920,7 @@
         <v>0</v>
       </c>
       <c r="F175">
-        <v>0.8088301824757718</v>
+        <v>0.8067191612749736</v>
       </c>
       <c r="G175">
         <v>0</v>
@@ -5929,7 +5929,7 @@
         <v>0.9</v>
       </c>
       <c r="I175">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="176" spans="1:9">
@@ -5952,13 +5952,13 @@
         <v>0</v>
       </c>
       <c r="G176">
-        <v>1.314701839907713</v>
+        <v>1.313011778265744</v>
       </c>
       <c r="H176">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I176">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="177" spans="1:9">
@@ -5981,13 +5981,13 @@
         <v>0</v>
       </c>
       <c r="G177">
-        <v>1.314701839907713</v>
+        <v>1.313011778265744</v>
       </c>
       <c r="H177">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I177">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="178" spans="1:9">
@@ -6010,13 +6010,13 @@
         <v>0</v>
       </c>
       <c r="G178">
-        <v>1.029582497201481</v>
+        <v>1.026895319439506</v>
       </c>
       <c r="H178">
         <v>0.9</v>
       </c>
       <c r="I178">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="179" spans="1:9">
@@ -6042,10 +6042,10 @@
         <v>0</v>
       </c>
       <c r="H179">
-        <v>0.6795911918746134</v>
+        <v>0.6785064012966276</v>
       </c>
       <c r="I179">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="180" spans="1:9">
@@ -6071,10 +6071,10 @@
         <v>0</v>
       </c>
       <c r="H180">
-        <v>0.6795911918746134</v>
+        <v>0.6785064012966276</v>
       </c>
       <c r="I180">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="181" spans="1:9">
@@ -6094,7 +6094,7 @@
         <v>0</v>
       </c>
       <c r="F181">
-        <v>9.270173771649674</v>
+        <v>9.245978911231461</v>
       </c>
       <c r="G181">
         <v>0</v>
@@ -6103,7 +6103,7 @@
         <v>0.9</v>
       </c>
       <c r="I181">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="182" spans="1:9">
@@ -6114,7 +6114,7 @@
         <v>10</v>
       </c>
       <c r="C182" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D182">
         <v>0</v>
@@ -6123,16 +6123,16 @@
         <v>0</v>
       </c>
       <c r="F182">
-        <v>0</v>
+        <v>2.303712824888164</v>
       </c>
       <c r="G182">
-        <v>2.306678081364841</v>
+        <v>0</v>
       </c>
       <c r="H182">
-        <v>0.7171704480218883</v>
+        <v>0.7313302934646828</v>
       </c>
       <c r="I182">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="183" spans="1:9">
@@ -6143,7 +6143,7 @@
         <v>12</v>
       </c>
       <c r="C183" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D183">
         <v>0</v>
@@ -6152,16 +6152,16 @@
         <v>0</v>
       </c>
       <c r="F183">
-        <v>0</v>
+        <v>2.303712824888164</v>
       </c>
       <c r="G183">
-        <v>2.306678081364841</v>
+        <v>0</v>
       </c>
       <c r="H183">
-        <v>0.7171704480218883</v>
+        <v>0.7313302934646828</v>
       </c>
       <c r="I183">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="184" spans="1:9">
@@ -6181,7 +6181,7 @@
         <v>0</v>
       </c>
       <c r="F184">
-        <v>1.806428885364793</v>
+        <v>1.801714163093838</v>
       </c>
       <c r="G184">
         <v>0</v>
@@ -6190,7 +6190,7 @@
         <v>0.9</v>
       </c>
       <c r="I184">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="185" spans="1:9">
@@ -6216,10 +6216,10 @@
         <v>0</v>
       </c>
       <c r="H185">
-        <v>0.6751324872921075</v>
+        <v>0.6790690123961114</v>
       </c>
       <c r="I185">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="186" spans="1:9">
@@ -6245,10 +6245,10 @@
         <v>0</v>
       </c>
       <c r="H186">
-        <v>0.6751324872921075</v>
+        <v>0.6790690123961114</v>
       </c>
       <c r="I186">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="187" spans="1:9">
@@ -6271,13 +6271,13 @@
         <v>0</v>
       </c>
       <c r="G187">
-        <v>0.9095525618320601</v>
+        <v>0.9071786584060151</v>
       </c>
       <c r="H187">
         <v>0.9</v>
       </c>
       <c r="I187">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="188" spans="1:9">
@@ -6297,16 +6297,16 @@
         <v>0</v>
       </c>
       <c r="F188">
-        <v>1.388750617834939</v>
+        <v>1.386351188420837</v>
       </c>
       <c r="G188">
-        <v>1.388750617834939</v>
+        <v>1.386351188420837</v>
       </c>
       <c r="H188">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I188">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="189" spans="1:9">
@@ -6326,16 +6326,16 @@
         <v>0</v>
       </c>
       <c r="F189">
-        <v>1.388750617834939</v>
+        <v>1.386351188420837</v>
       </c>
       <c r="G189">
-        <v>1.388750617834939</v>
+        <v>1.386351188420837</v>
       </c>
       <c r="H189">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I189">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="190" spans="1:9">
@@ -6355,7 +6355,7 @@
         <v>0</v>
       </c>
       <c r="F190">
-        <v>0.8088301824757718</v>
+        <v>0.8067191612749736</v>
       </c>
       <c r="G190">
         <v>0</v>
@@ -6364,7 +6364,7 @@
         <v>0.9</v>
       </c>
       <c r="I190">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="191" spans="1:9">
@@ -6387,13 +6387,13 @@
         <v>0</v>
       </c>
       <c r="G191">
-        <v>1.314701839907713</v>
+        <v>1.313011778265744</v>
       </c>
       <c r="H191">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I191">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="192" spans="1:9">
@@ -6416,13 +6416,13 @@
         <v>0</v>
       </c>
       <c r="G192">
-        <v>1.314701839907713</v>
+        <v>1.313011778265744</v>
       </c>
       <c r="H192">
-        <v>0.6948796794294304</v>
+        <v>0.7138742859435663</v>
       </c>
       <c r="I192">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="193" spans="1:9">
@@ -6445,13 +6445,13 @@
         <v>0</v>
       </c>
       <c r="G193">
-        <v>1.029582497201481</v>
+        <v>1.026895319439506</v>
       </c>
       <c r="H193">
         <v>0.9</v>
       </c>
       <c r="I193">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="194" spans="1:9">
@@ -6477,10 +6477,10 @@
         <v>0</v>
       </c>
       <c r="H194">
-        <v>0.6994687982605935</v>
+        <v>0.7132828385507737</v>
       </c>
       <c r="I194">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="195" spans="1:9">
@@ -6506,10 +6506,10 @@
         <v>0</v>
       </c>
       <c r="H195">
-        <v>0.6994687982605935</v>
+        <v>0.7132828385507737</v>
       </c>
       <c r="I195">
-        <v>0.1774002065716946</v>
+        <v>0.1772186337722917</v>
       </c>
     </row>
     <row r="196" spans="1:9">
@@ -6529,7 +6529,7 @@
         <v>0</v>
       </c>
       <c r="F196">
-        <v>8.831430106227877</v>
+        <v>8.808380352903214</v>
       </c>
       <c r="G196">
         <v>0</v>
@@ -6538,7 +6538,7 @@
         <v>0.9</v>
       </c>
       <c r="I196">
-        <v>0.1453586326313147</v>
+        <v>0.1450425316067563</v>
       </c>
     </row>
     <row r="197" spans="1:9">
@@ -6558,16 +6558,16 @@
         <v>0</v>
       </c>
       <c r="F197">
-        <v>2.664478377616962</v>
+        <v>2.664276551727783</v>
       </c>
       <c r="G197">
         <v>0</v>
       </c>
       <c r="H197">
-        <v>0.7665750039208149</v>
+        <v>0.7653298680559651</v>
       </c>
       <c r="I197">
-        <v>0.1986319186045138</v>
+        <v>0.1986203095082267</v>
       </c>
     </row>
     <row r="198" spans="1:9">
@@ -6587,16 +6587,16 @@
         <v>0</v>
       </c>
       <c r="F198">
-        <v>2.664478377616962</v>
+        <v>2.664276551727783</v>
       </c>
       <c r="G198">
         <v>0</v>
       </c>
       <c r="H198">
-        <v>0.7665750039208149</v>
+        <v>0.7653298680559651</v>
       </c>
       <c r="I198">
-        <v>0.1986319186045138</v>
+        <v>0.1986203095082267</v>
       </c>
     </row>
     <row r="199" spans="1:9">
@@ -6616,7 +6616,7 @@
         <v>0</v>
       </c>
       <c r="F199">
-        <v>1.930213251555818</v>
+        <v>1.92773469264805</v>
       </c>
       <c r="G199">
         <v>0</v>
@@ -6625,7 +6625,7 @@
         <v>0.9</v>
       </c>
       <c r="I199">
-        <v>0.1535602524005467</v>
+        <v>0.1533978527327384</v>
       </c>
     </row>
     <row r="200" spans="1:9">
@@ -6648,13 +6648,13 @@
         <v>0</v>
       </c>
       <c r="G200">
-        <v>1.341587899718641</v>
+        <v>1.341486278638489</v>
       </c>
       <c r="H200">
-        <v>0.7404437426436037</v>
+        <v>0.745281166398304</v>
       </c>
       <c r="I200">
-        <v>0.1986319186045138</v>
+        <v>0.1986203095082267</v>
       </c>
     </row>
     <row r="201" spans="1:9">
@@ -6677,13 +6677,13 @@
         <v>0</v>
       </c>
       <c r="G201">
-        <v>1.341587899718641</v>
+        <v>1.341486278638489</v>
       </c>
       <c r="H201">
-        <v>0.7404437426436037</v>
+        <v>0.745281166398304</v>
       </c>
       <c r="I201">
-        <v>0.1986319186045138</v>
+        <v>0.1986203095082267</v>
       </c>
     </row>
     <row r="202" spans="1:9">
@@ -6706,13 +6706,13 @@
         <v>0</v>
       </c>
       <c r="G202">
-        <v>0.9718790604260348</v>
+        <v>0.9706310845868109</v>
       </c>
       <c r="H202">
         <v>0.9</v>
       </c>
       <c r="I202">
-        <v>0.1535602524005467</v>
+        <v>0.1533978527327384</v>
       </c>
     </row>
     <row r="203" spans="1:9">
@@ -6732,16 +6732,16 @@
         <v>0</v>
       </c>
       <c r="F203">
-        <v>1.193022625928321</v>
+        <v>1.192932258202198</v>
       </c>
       <c r="G203">
         <v>0</v>
       </c>
       <c r="H203">
-        <v>0.7404437426436037</v>
+        <v>0.745281166398304</v>
       </c>
       <c r="I203">
-        <v>0.1986319186045138</v>
+        <v>0.1986203095082267</v>
       </c>
     </row>
     <row r="204" spans="1:9">
@@ -6761,16 +6761,16 @@
         <v>0</v>
       </c>
       <c r="F204">
-        <v>1.193022625928321</v>
+        <v>1.192932258202198</v>
       </c>
       <c r="G204">
         <v>0</v>
       </c>
       <c r="H204">
-        <v>0.7404437426436037</v>
+        <v>0.745281166398304</v>
       </c>
       <c r="I204">
-        <v>0.1986319186045138</v>
+        <v>0.1986203095082267</v>
       </c>
     </row>
     <row r="205" spans="1:9">
@@ -6790,7 +6790,7 @@
         <v>0</v>
       </c>
       <c r="F205">
-        <v>0.864254745438136</v>
+        <v>0.8631449684245549</v>
       </c>
       <c r="G205">
         <v>0</v>
@@ -6799,7 +6799,7 @@
         <v>0.9</v>
       </c>
       <c r="I205">
-        <v>0.1535602524005467</v>
+        <v>0.1533978527327384</v>
       </c>
     </row>
     <row r="206" spans="1:9">
@@ -6822,13 +6822,13 @@
         <v>0</v>
       </c>
       <c r="G206">
-        <v>1.518631773435263</v>
+        <v>1.518516741836364</v>
       </c>
       <c r="H206">
-        <v>0.7621012471009998</v>
+        <v>0.7834801040507973</v>
       </c>
       <c r="I206">
-        <v>0.1986319186045138</v>
+        <v>0.1986203095082267</v>
       </c>
     </row>
     <row r="207" spans="1:9">
@@ -6851,13 +6851,13 @@
         <v>0</v>
       </c>
       <c r="G207">
-        <v>1.518631773435263</v>
+        <v>1.518516741836364</v>
       </c>
       <c r="H207">
-        <v>0.7621012471009998</v>
+        <v>0.7834801040507973</v>
       </c>
       <c r="I207">
-        <v>0.1986319186045138</v>
+        <v>0.1986203095082267</v>
       </c>
     </row>
     <row r="208" spans="1:9">
@@ -6880,13 +6880,13 @@
         <v>0</v>
       </c>
       <c r="G208">
-        <v>1.100133969163645</v>
+        <v>1.098721303051851</v>
       </c>
       <c r="H208">
         <v>0.9</v>
       </c>
       <c r="I208">
-        <v>0.1535602524005467</v>
+        <v>0.1533978527327384</v>
       </c>
     </row>
     <row r="209" spans="1:9">
@@ -6897,7 +6897,7 @@
         <v>10</v>
       </c>
       <c r="C209" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="D209">
         <v>0</v>
@@ -6909,13 +6909,13 @@
         <v>0</v>
       </c>
       <c r="G209">
-        <v>0</v>
+        <v>2.866922508804143</v>
       </c>
       <c r="H209">
-        <v>0.78899683100665</v>
+        <v>0.8045563898460469</v>
       </c>
       <c r="I209">
-        <v>0.1986319186045138</v>
+        <v>0.1986203095082267</v>
       </c>
     </row>
     <row r="210" spans="1:9">
@@ -6938,13 +6938,13 @@
         <v>0</v>
       </c>
       <c r="G210">
-        <v>0</v>
+        <v>2.866922508804143</v>
       </c>
       <c r="H210">
-        <v>0.78899683100665</v>
+        <v>0.8045563898460469</v>
       </c>
       <c r="I210">
-        <v>0.1986319186045138</v>
+        <v>0.1986203095082267</v>
       </c>
     </row>
     <row r="211" spans="1:9">
@@ -6973,7 +6973,7 @@
         <v>0.9</v>
       </c>
       <c r="I211">
-        <v>0.1535602524005467</v>
+        <v>0.1533978527327384</v>
       </c>
     </row>
     <row r="212" spans="1:9">
@@ -6999,10 +6999,10 @@
         <v>0</v>
       </c>
       <c r="H212">
-        <v>0.7621012471009998</v>
+        <v>0.7834801040507973</v>
       </c>
       <c r="I212">
-        <v>0.1986319186045138</v>
+        <v>0.1986203095082267</v>
       </c>
     </row>
     <row r="213" spans="1:9">
@@ -7028,10 +7028,10 @@
         <v>0</v>
       </c>
       <c r="H213">
-        <v>0.7621012471009998</v>
+        <v>0.7834801040507973</v>
       </c>
       <c r="I213">
-        <v>0.1986319186045138</v>
+        <v>0.1986203095082267</v>
       </c>
     </row>
     <row r="214" spans="1:9">
@@ -7054,13 +7054,13 @@
         <v>0</v>
       </c>
       <c r="G214">
-        <v>0.9718790604260348</v>
+        <v>0.9706310845868109</v>
       </c>
       <c r="H214">
         <v>0.9</v>
       </c>
       <c r="I214">
-        <v>0.1535602524005467</v>
+        <v>0.1533978527327384</v>
       </c>
     </row>
     <row r="215" spans="1:9">
@@ -7080,16 +7080,16 @@
         <v>0</v>
       </c>
       <c r="F215">
-        <v>1.231526879377206</v>
+        <v>1.23143359507452</v>
       </c>
       <c r="G215">
         <v>0</v>
       </c>
       <c r="H215">
-        <v>0.7621012471009998</v>
+        <v>0.7834801040507973</v>
       </c>
       <c r="I215">
-        <v>0.1986319186045138</v>
+        <v>0.1986203095082267</v>
       </c>
     </row>
     <row r="216" spans="1:9">
@@ -7109,16 +7109,16 @@
         <v>0</v>
       </c>
       <c r="F216">
-        <v>1.231526879377206</v>
+        <v>1.23143359507452</v>
       </c>
       <c r="G216">
         <v>0</v>
       </c>
       <c r="H216">
-        <v>0.7621012471009998</v>
+        <v>0.7834801040507973</v>
       </c>
       <c r="I216">
-        <v>0.1986319186045138</v>
+        <v>0.1986203095082267</v>
       </c>
     </row>
     <row r="217" spans="1:9">
@@ -7147,7 +7147,7 @@
         <v>0.9</v>
       </c>
       <c r="I217">
-        <v>0.1535602524005467</v>
+        <v>0.1533978527327384</v>
       </c>
     </row>
     <row r="218" spans="1:9">
@@ -7158,7 +7158,7 @@
         <v>10</v>
       </c>
       <c r="C218" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D218">
         <v>0</v>
@@ -7167,16 +7167,16 @@
         <v>0</v>
       </c>
       <c r="F218">
-        <v>0</v>
+        <v>1.518516741836363</v>
       </c>
       <c r="G218">
         <v>0</v>
       </c>
       <c r="H218">
-        <v>0.7621012471009998</v>
+        <v>0.7834801040507973</v>
       </c>
       <c r="I218">
-        <v>0.1986319186045138</v>
+        <v>0.1986203095082267</v>
       </c>
     </row>
     <row r="219" spans="1:9">
@@ -7187,7 +7187,7 @@
         <v>12</v>
       </c>
       <c r="C219" t="s">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="D219">
         <v>0</v>
@@ -7196,16 +7196,16 @@
         <v>0</v>
       </c>
       <c r="F219">
-        <v>0</v>
+        <v>1.518516741836363</v>
       </c>
       <c r="G219">
         <v>0</v>
       </c>
       <c r="H219">
-        <v>0.7621012471009998</v>
+        <v>0.7834801040507973</v>
       </c>
       <c r="I219">
-        <v>0.1986319186045138</v>
+        <v>0.1986203095082267</v>
       </c>
     </row>
     <row r="220" spans="1:9">
@@ -7234,7 +7234,7 @@
         <v>0.9</v>
       </c>
       <c r="I220">
-        <v>0.1535602524005467</v>
+        <v>0.1533978527327384</v>
       </c>
     </row>
     <row r="221" spans="1:9">
@@ -7260,10 +7260,10 @@
         <v>0</v>
       </c>
       <c r="H221">
-        <v>0.3257265520050494</v>
+        <v>0.325230629628477</v>
       </c>
       <c r="I221">
-        <v>0.1957745045587984</v>
+        <v>0.1955511814377309</v>
       </c>
     </row>
     <row r="222" spans="1:9">
@@ -7289,10 +7289,10 @@
         <v>0</v>
       </c>
       <c r="H222">
-        <v>0.3257265520050494</v>
+        <v>0.325230629628477</v>
       </c>
       <c r="I222">
-        <v>0.1957745045587984</v>
+        <v>0.1955511814377309</v>
       </c>
     </row>
     <row r="223" spans="1:9">
@@ -7312,16 +7312,16 @@
         <v>0</v>
       </c>
       <c r="F223">
-        <v>0.00544137499505562</v>
+        <v>0.005426460371284084</v>
       </c>
       <c r="G223">
         <v>0</v>
       </c>
       <c r="H223">
-        <v>0.798126902270676</v>
+        <v>0.7960156053668845</v>
       </c>
       <c r="I223">
-        <v>0.1510535043242025</v>
+        <v>0.1507112310599028</v>
       </c>
     </row>
     <row r="224" spans="1:9">
@@ -7332,7 +7332,7 @@
         <v>10</v>
       </c>
       <c r="C224" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="D224">
         <v>0</v>
@@ -7347,10 +7347,10 @@
         <v>0</v>
       </c>
       <c r="H224">
-        <v>0.7672628912150288</v>
+        <v>0.7729889724690531</v>
       </c>
       <c r="I224">
-        <v>0.1986319186045138</v>
+        <v>0.1986203095082267</v>
       </c>
     </row>
     <row r="225" spans="1:9">
@@ -7376,10 +7376,10 @@
         <v>0</v>
       </c>
       <c r="H225">
-        <v>0.7672628912150288</v>
+        <v>0.7729889724690531</v>
       </c>
       <c r="I225">
-        <v>0.1986319186045138</v>
+        <v>0.1986203095082267</v>
       </c>
     </row>
     <row r="226" spans="1:9">
@@ -7399,7 +7399,7 @@
         <v>0</v>
       </c>
       <c r="F226">
-        <v>0.5861669328440866</v>
+        <v>0.5854142443669621</v>
       </c>
       <c r="G226">
         <v>0</v>
@@ -7408,7 +7408,7 @@
         <v>0.9</v>
       </c>
       <c r="I226">
-        <v>0.1535602524005467</v>
+        <v>0.1533978527327384</v>
       </c>
     </row>
   </sheetData>

</xml_diff>